<commit_message>
Record traceability register commit
Record the implementation commit for CHG-0001 in the traceability register.

Implementation commit:
04e8e72054f693b237cd7f0ad4e3755eb08d2d91

This is a metadata-only traceability update.
No scientific, numerical, API or ABI behaviour is changed.
</commit_message>
<xml_diff>
--- a/planning/traceability/MOHID-NG_Traceability_Register.xlsx
+++ b/planning/traceability/MOHID-NG_Traceability_Register.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04-Test\home\jflavio\Programas\MohidNG\planning\traceability\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{326FA6ED-C6CC-4B96-830B-1D52D5F9F90E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D09DC598-BEFA-4A28-A462-C7275A755A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="570">
   <si>
     <t>MOHID-NG Traceability and Change-Management Register</t>
   </si>
@@ -1751,6 +1751,9 @@
   </si>
   <si>
     <t>p0/traceability-register</t>
+  </si>
+  <si>
+    <t>04e8e72054f693b237cd7f0ad4e3755eb08d2d91</t>
   </si>
 </sst>
 </file>
@@ -1871,6 +1874,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1889,17 +1898,67 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="35">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD9EAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1980,62 +2039,6 @@
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFD9EAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2279,33 +2282,33 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ChangeRegisterTable" displayName="ChangeRegisterTable" ref="A1:Y2" totalsRowShown="0" headerRowDxfId="26" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ChangeRegisterTable" displayName="ChangeRegisterTable" ref="A1:Y2" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="CHG_ID" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Data" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Título" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Categoria" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Status" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Prioridade" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Responsável" dataDxfId="19"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Fonte/Justificativa" dataDxfId="18"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="REQ_IDs" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ADR_IDs" dataDxfId="16"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Arquivos/paths" dataDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Resumo da alteração" dataDxfId="14"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Razão" dataDxfId="13"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Testes/Gates" dataDxfId="12"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="EVID_IDs" dataDxfId="11"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Branch" dataDxfId="10"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Commit" dataDxfId="9"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="PR" dataDxfId="8"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Release" dataDxfId="7"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Impacto científico" dataDxfId="6"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Impacto numérico" dataDxfId="5"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Impacto API/ABI" dataDxfId="4"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0100-000017000000}" name="Documentação atualizada" dataDxfId="3"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0100-000018000000}" name="Compatibilidade/risco" dataDxfId="2"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0100-000019000000}" name="Observações" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="CHG_ID" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Data" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Título" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Categoria" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Status" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Prioridade" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Responsável" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Fonte/Justificativa" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="REQ_IDs" dataDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ADR_IDs" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Arquivos/paths" dataDxfId="22"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Resumo da alteração" dataDxfId="21"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Razão" dataDxfId="20"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Testes/Gates" dataDxfId="19"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="EVID_IDs" dataDxfId="18"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Branch" dataDxfId="17"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Commit" dataDxfId="16"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="PR" dataDxfId="15"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Release" dataDxfId="14"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Impacto científico" dataDxfId="13"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Impacto numérico" dataDxfId="12"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Impacto API/ABI" dataDxfId="11"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0100-000017000000}" name="Documentação atualizada" dataDxfId="10"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0100-000018000000}" name="Compatibilidade/risco" dataDxfId="9"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0100-000019000000}" name="Observações" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2637,16 +2640,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2"/>
@@ -2795,16 +2798,16 @@
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="15">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="5" t="s">
@@ -2943,38 +2946,38 @@
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:8" ht="15">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
+      <c r="A26" s="16"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16"/>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2"/>
@@ -2987,58 +2990,58 @@
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:8" ht="15">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -5099,38 +5102,38 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="13" t="s">
         <v>567</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5152,16 +5155,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
     </row>
     <row r="3" spans="1:8" ht="15">
       <c r="A3" s="1" t="s">
@@ -5267,68 +5270,68 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="15">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6094,13 +6097,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D100">
-    <cfRule type="expression" dxfId="34" priority="1">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>D2="Concluído"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>D2="Em andamento"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="3">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>D2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6144,7 +6147,7 @@
     <col min="25" max="25" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="17" customFormat="1" ht="30">
+    <row r="1" spans="1:25" s="11" customFormat="1" ht="30">
       <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
@@ -6225,7 +6228,7 @@
       <c r="A2" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="B2" s="18">
+      <c r="B2" s="12">
         <v>46273</v>
       </c>
       <c r="C2" s="8" t="s">
@@ -6264,7 +6267,9 @@
       <c r="P2" s="8" t="s">
         <v>568</v>
       </c>
-      <c r="Q2" s="8"/>
+      <c r="Q2" s="8" t="s">
+        <v>569</v>
+      </c>
       <c r="R2" s="8"/>
       <c r="S2" s="8"/>
       <c r="T2" s="8" t="s">
@@ -22426,19 +22431,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F500">
-    <cfRule type="expression" dxfId="31" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>F2="REUSE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>F2="REFACTOR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>F2="REPLACE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>F2="REMOVE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>F2="INVESTIGATE"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Record pull request in traceability register
Record PR #1 for CHG-0001 in the MOHID-NG traceability register.

This is a metadata-only traceability update.

No scientific, numerical, API, ABI or runtime behaviour is changed.
</commit_message>
<xml_diff>
--- a/planning/traceability/MOHID-NG_Traceability_Register.xlsx
+++ b/planning/traceability/MOHID-NG_Traceability_Register.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04-Test\home\jflavio\Programas\MohidNG\planning\traceability\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D09DC598-BEFA-4A28-A462-C7275A755A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B3759A-1B7C-412D-8CD7-4E30AB05F12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="571">
   <si>
     <t>MOHID-NG Traceability and Change-Management Register</t>
   </si>
@@ -1754,6 +1754,9 @@
   </si>
   <si>
     <t>04e8e72054f693b237cd7f0ad4e3755eb08d2d91</t>
+  </si>
+  <si>
+    <t>#1</t>
   </si>
 </sst>
 </file>
@@ -1844,7 +1847,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1879,6 +1882,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1981,7 +1987,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2640,16 +2646,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2"/>
@@ -2798,16 +2804,16 @@
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="15">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="5" t="s">
@@ -2946,38 +2952,38 @@
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:8" ht="15">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="16"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2"/>
@@ -2990,58 +2996,58 @@
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:8" ht="15">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="13"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -5102,38 +5108,38 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="14" t="s">
         <v>567</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5155,16 +5161,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="3" spans="1:8" ht="15">
       <c r="A3" s="1" t="s">
@@ -5270,68 +5276,68 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="15">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6270,7 +6276,9 @@
       <c r="Q2" s="8" t="s">
         <v>569</v>
       </c>
-      <c r="R2" s="8"/>
+      <c r="R2" s="13" t="s">
+        <v>570</v>
+      </c>
       <c r="S2" s="8"/>
       <c r="T2" s="8" t="s">
         <v>157</v>

</xml_diff>

<commit_message>
Define MOHID-NG license as MPL-2.0
Adopt Mozilla Public License 2.0 for MOHID-NG and record the resolution of D-OPEN-11 in the traceability register.
</commit_message>
<xml_diff>
--- a/planning/traceability/MOHID-NG_Traceability_Register.xlsx
+++ b/planning/traceability/MOHID-NG_Traceability_Register.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04-Test\home\jflavio\Programas\MohidNG\planning\traceability\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B3759A-1B7C-412D-8CD7-4E30AB05F12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03CA43C5-D21A-42AA-8BFD-A9E910DD368F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_README" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="574">
   <si>
     <t>MOHID-NG Traceability and Change-Management Register</t>
   </si>
@@ -1757,6 +1757,15 @@
   </si>
   <si>
     <t>#1</t>
+  </si>
+  <si>
+    <t>Copyleft em nível de arquivo, preservando abertas as modificações distribuídas do núcleo do MOHID-NG e permitindo que aplicações, extensões e componentes independentes utilizem outras licenças.</t>
+  </si>
+  <si>
+    <t>Licença adotada: Mozilla Public License 2.0 (MPL-2.0). Ver arquivo LICENSE.</t>
+  </si>
+  <si>
+    <t>Definida</t>
   </si>
 </sst>
 </file>
@@ -1847,7 +1856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1904,11 +1913,52 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="39">
+    <dxf>
+      <alignment horizontal="general" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2288,33 +2338,33 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ChangeRegisterTable" displayName="ChangeRegisterTable" ref="A1:Y2" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ChangeRegisterTable" displayName="ChangeRegisterTable" ref="A1:Y2" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="CHG_ID" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Data" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Título" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Categoria" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Status" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Prioridade" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Responsável" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Fonte/Justificativa" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="REQ_IDs" dataDxfId="24"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ADR_IDs" dataDxfId="23"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Arquivos/paths" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Resumo da alteração" dataDxfId="21"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Razão" dataDxfId="20"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Testes/Gates" dataDxfId="19"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="EVID_IDs" dataDxfId="18"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Branch" dataDxfId="17"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Commit" dataDxfId="16"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="PR" dataDxfId="15"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Release" dataDxfId="14"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Impacto científico" dataDxfId="13"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Impacto numérico" dataDxfId="12"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Impacto API/ABI" dataDxfId="11"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0100-000017000000}" name="Documentação atualizada" dataDxfId="10"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0100-000018000000}" name="Compatibilidade/risco" dataDxfId="9"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0100-000019000000}" name="Observações" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="CHG_ID" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Data" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Título" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Categoria" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Status" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Prioridade" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Responsável" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Fonte/Justificativa" dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="REQ_IDs" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ADR_IDs" dataDxfId="27"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Arquivos/paths" dataDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Resumo da alteração" dataDxfId="25"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Razão" dataDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Testes/Gates" dataDxfId="23"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="EVID_IDs" dataDxfId="22"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Branch" dataDxfId="21"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Commit" dataDxfId="20"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="PR" dataDxfId="19"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Release" dataDxfId="18"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Impacto científico" dataDxfId="17"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Impacto numérico" dataDxfId="16"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Impacto API/ABI" dataDxfId="15"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0100-000017000000}" name="Documentação atualizada" dataDxfId="14"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0100-000018000000}" name="Compatibilidade/risco" dataDxfId="13"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0100-000019000000}" name="Observações" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2367,15 +2417,15 @@
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Record_ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Tipo"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Decisão/Título"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Status"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Fonte"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Decisão/Título" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Status" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Fonte" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="REQ_IDs"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="ADR_file"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Supersedes"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Racional/Evidência"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" name="Responsável"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Data decisão"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Data decisão" dataDxfId="3"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" name="Observações"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -5272,7 +5322,7 @@
       </c>
       <c r="B9" s="2">
         <f>COUNTIF('06_Decisions_ADRs'!D2:D200,"Em aberto")</f>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15">
@@ -6103,13 +6153,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D100">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>D2="Concluído"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>D2="Em andamento"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>D2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22439,19 +22489,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F500">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="8" priority="1">
       <formula>F2="REUSE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="7" priority="2">
       <formula>F2="REFACTOR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="6" priority="3">
       <formula>F2="REPLACE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>F2="REMOVE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>F2="INVESTIGATE"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24194,14 +24244,17 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L200"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="66" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="3" max="3" width="66" style="24" customWidth="1"/>
+    <col min="4" max="4" width="22" style="22" customWidth="1"/>
+    <col min="5" max="5" width="16" style="22" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="34" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
@@ -24218,13 +24271,13 @@
       <c r="B1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="23" t="s">
         <v>369</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="7" t="s">
         <v>60</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -24259,10 +24312,10 @@
       <c r="C2" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F2" s="3"/>
@@ -24270,7 +24323,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="4"/>
+      <c r="K2" s="20"/>
       <c r="L2" s="3"/>
     </row>
     <row r="3" spans="1:12">
@@ -24283,10 +24336,10 @@
       <c r="C3" s="3" t="s">
         <v>380</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F3" s="3"/>
@@ -24294,7 +24347,7 @@
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="4"/>
+      <c r="K3" s="20"/>
       <c r="L3" s="3"/>
     </row>
     <row r="4" spans="1:12">
@@ -24307,10 +24360,10 @@
       <c r="C4" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F4" s="3"/>
@@ -24318,7 +24371,7 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
-      <c r="K4" s="4"/>
+      <c r="K4" s="20"/>
       <c r="L4" s="3"/>
     </row>
     <row r="5" spans="1:12">
@@ -24331,10 +24384,10 @@
       <c r="C5" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="8" t="s">
         <v>378</v>
       </c>
       <c r="F5" s="3"/>
@@ -24342,7 +24395,7 @@
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
-      <c r="K5" s="4"/>
+      <c r="K5" s="20"/>
       <c r="L5" s="3"/>
     </row>
     <row r="6" spans="1:12" ht="28.5">
@@ -24355,10 +24408,10 @@
       <c r="C6" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F6" s="3"/>
@@ -24366,7 +24419,7 @@
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
-      <c r="K6" s="4"/>
+      <c r="K6" s="20"/>
       <c r="L6" s="3"/>
     </row>
     <row r="7" spans="1:12">
@@ -24379,10 +24432,10 @@
       <c r="C7" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F7" s="3"/>
@@ -24390,7 +24443,7 @@
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="20"/>
       <c r="L7" s="3"/>
     </row>
     <row r="8" spans="1:12">
@@ -24403,10 +24456,10 @@
       <c r="C8" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F8" s="3"/>
@@ -24414,7 +24467,7 @@
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
-      <c r="K8" s="4"/>
+      <c r="K8" s="20"/>
       <c r="L8" s="3"/>
     </row>
     <row r="9" spans="1:12">
@@ -24427,10 +24480,10 @@
       <c r="C9" s="3" t="s">
         <v>392</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F9" s="3"/>
@@ -24438,7 +24491,7 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
-      <c r="K9" s="4"/>
+      <c r="K9" s="20"/>
       <c r="L9" s="3"/>
     </row>
     <row r="10" spans="1:12">
@@ -24451,10 +24504,10 @@
       <c r="C10" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F10" s="3"/>
@@ -24462,7 +24515,7 @@
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
-      <c r="K10" s="4"/>
+      <c r="K10" s="20"/>
       <c r="L10" s="3"/>
     </row>
     <row r="11" spans="1:12">
@@ -24475,10 +24528,10 @@
       <c r="C11" s="3" t="s">
         <v>396</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F11" s="3"/>
@@ -24486,32 +24539,40 @@
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
-      <c r="K11" s="4"/>
+      <c r="K11" s="20"/>
       <c r="L11" s="3"/>
     </row>
-    <row r="12" spans="1:12">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:12" s="29" customFormat="1" ht="67.5" customHeight="1">
+      <c r="A12" s="25" t="s">
         <v>397</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="25" t="s">
         <v>375</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="26" t="s">
         <v>398</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="E12" s="3" t="s">
+      <c r="D12" s="27" t="s">
+        <v>573</v>
+      </c>
+      <c r="E12" s="27" t="s">
         <v>378</v>
       </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="3"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="27" t="s">
+        <v>571</v>
+      </c>
+      <c r="J12" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="K12" s="28">
+        <v>46273</v>
+      </c>
+      <c r="L12" s="27" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="3" t="s">
@@ -24523,10 +24584,10 @@
       <c r="C13" s="3" t="s">
         <v>400</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F13" s="3"/>
@@ -24534,7 +24595,7 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
-      <c r="K13" s="4"/>
+      <c r="K13" s="20"/>
       <c r="L13" s="3"/>
     </row>
     <row r="14" spans="1:12" ht="28.5">
@@ -24547,10 +24608,10 @@
       <c r="C14" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F14" s="3"/>
@@ -24558,7 +24619,7 @@
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
-      <c r="K14" s="4"/>
+      <c r="K14" s="20"/>
       <c r="L14" s="3"/>
     </row>
     <row r="15" spans="1:12" ht="28.5">
@@ -24571,10 +24632,10 @@
       <c r="C15" s="3" t="s">
         <v>404</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F15" s="3"/>
@@ -24582,7 +24643,7 @@
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
-      <c r="K15" s="4"/>
+      <c r="K15" s="20"/>
       <c r="L15" s="3"/>
     </row>
     <row r="16" spans="1:12">
@@ -24595,10 +24656,10 @@
       <c r="C16" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F16" s="3"/>
@@ -24606,7 +24667,7 @@
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
-      <c r="K16" s="4"/>
+      <c r="K16" s="20"/>
       <c r="L16" s="3"/>
     </row>
     <row r="17" spans="1:12">
@@ -24619,10 +24680,10 @@
       <c r="C17" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="21" t="s">
         <v>378</v>
       </c>
       <c r="F17" s="3"/>
@@ -24630,7 +24691,7 @@
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
-      <c r="K17" s="4"/>
+      <c r="K17" s="20"/>
       <c r="L17" s="3"/>
     </row>
     <row r="18" spans="1:12" ht="28.5">
@@ -24641,10 +24702,10 @@
       <c r="C18" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F18" s="3"/>
@@ -24652,7 +24713,7 @@
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
-      <c r="K18" s="4"/>
+      <c r="K18" s="20"/>
       <c r="L18" s="3" t="s">
         <v>413</v>
       </c>
@@ -24665,10 +24726,10 @@
       <c r="C19" s="3" t="s">
         <v>414</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F19" s="3"/>
@@ -24676,7 +24737,7 @@
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
-      <c r="K19" s="4"/>
+      <c r="K19" s="20"/>
       <c r="L19" s="3" t="s">
         <v>413</v>
       </c>
@@ -24689,10 +24750,10 @@
       <c r="C20" s="3" t="s">
         <v>415</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F20" s="3"/>
@@ -24700,7 +24761,7 @@
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
-      <c r="K20" s="4"/>
+      <c r="K20" s="20"/>
       <c r="L20" s="3" t="s">
         <v>413</v>
       </c>
@@ -24713,10 +24774,10 @@
       <c r="C21" s="3" t="s">
         <v>416</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F21" s="3"/>
@@ -24724,7 +24785,7 @@
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
-      <c r="K21" s="4"/>
+      <c r="K21" s="20"/>
       <c r="L21" s="3" t="s">
         <v>413</v>
       </c>
@@ -24737,10 +24798,10 @@
       <c r="C22" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F22" s="3"/>
@@ -24748,7 +24809,7 @@
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
-      <c r="K22" s="4"/>
+      <c r="K22" s="20"/>
       <c r="L22" s="3" t="s">
         <v>413</v>
       </c>
@@ -24761,10 +24822,10 @@
       <c r="C23" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F23" s="3"/>
@@ -24772,7 +24833,7 @@
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
-      <c r="K23" s="4"/>
+      <c r="K23" s="20"/>
       <c r="L23" s="3" t="s">
         <v>413</v>
       </c>
@@ -24785,10 +24846,10 @@
       <c r="C24" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F24" s="3"/>
@@ -24796,7 +24857,7 @@
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
-      <c r="K24" s="4"/>
+      <c r="K24" s="20"/>
       <c r="L24" s="3" t="s">
         <v>413</v>
       </c>
@@ -24809,10 +24870,10 @@
       <c r="C25" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F25" s="3"/>
@@ -24820,7 +24881,7 @@
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
-      <c r="K25" s="4"/>
+      <c r="K25" s="20"/>
       <c r="L25" s="3" t="s">
         <v>413</v>
       </c>
@@ -24833,10 +24894,10 @@
       <c r="C26" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F26" s="3"/>
@@ -24844,7 +24905,7 @@
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
-      <c r="K26" s="4"/>
+      <c r="K26" s="20"/>
       <c r="L26" s="3" t="s">
         <v>413</v>
       </c>
@@ -24857,10 +24918,10 @@
       <c r="C27" s="3" t="s">
         <v>422</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="21" t="s">
         <v>412</v>
       </c>
       <c r="F27" s="3"/>
@@ -24868,7 +24929,7 @@
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
-      <c r="K27" s="4"/>
+      <c r="K27" s="20"/>
       <c r="L27" s="3" t="s">
         <v>413</v>
       </c>
@@ -25399,8 +25460,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="35" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Reorganização e otimização da infraestrutura CMake.
Alterações realizadas com assistência do Codex, a pedido do mantenedor, restritas aos arquivos de CMake e à infraestrutura de build. O objetivo foi simplificar e tornar mais consistente o processo de compilação, melhorar a organização das configurações de build e habilitar mecanismos apropriados de otimização de compilação. Não foram alterados modelos científicos, métodos numéricos ou funcionalidades do MOHID-NG. Ganhos efetivos de desempenho ainda não foram verificados por benchmark.
</commit_message>
<xml_diff>
--- a/planning/traceability/MOHID-NG_Traceability_Register.xlsx
+++ b/planning/traceability/MOHID-NG_Traceability_Register.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04-Test\home\jflavio\Programas\MohidNG\planning\traceability\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D0B1F4-3467-40D8-A4A2-C3D62607B983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6410E2F-2F10-47BD-AF1A-9C89167E39EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_README" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="592">
   <si>
     <t>MOHID-NG Traceability and Change-Management Register</t>
   </si>
@@ -1784,6 +1784,42 @@
   </si>
   <si>
     <t>Novas decisões de projeto que não sejam D-OPEN nem ADR formalizado usam DEC-xxxx.</t>
+  </si>
+  <si>
+    <t>Reorganização e otimização da infraestrutura Cmake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado </t>
+  </si>
+  <si>
+    <t>MOHID-NG System Definition v0.14, Item 6.8, Item 16.2 e Apêndice D.5</t>
+  </si>
+  <si>
+    <t>cmake/...</t>
+  </si>
+  <si>
+    <t>Reorganização da infraestrutura CMake para simplificar a compilação, melhorar a organização do  build e habilitar configurações apropriadas de otimização.</t>
+  </si>
+  <si>
+    <t>Facilitar a compilação e manutenção do projeto e permitir a utilização consistente das opções de  otimização previstas pelo sistema de build.</t>
+  </si>
+  <si>
+    <t>Configuração CMake e compilação verificadas.</t>
+  </si>
+  <si>
+    <t>Configuração e compilação bem-sucedidas após reorganização do CMake.</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>Baixo , alteração restrita à infraestrutura de build; requer verificação de compilação nos toolchains suportados.</t>
+  </si>
+  <si>
+    <t>Alteração restrita ao sistema de build, realizada com assistência do Codex a pedido do mantenedor. Não modifica modelos científicos, métodos numéricos ou comportamento funcional. Eventuais ganhos de desempenho dependem das configurações de compilação e ainda não foram verificados por benchmark.</t>
   </si>
 </sst>
 </file>
@@ -1874,7 +1910,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1949,11 +1985,23 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="49">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2009,6 +2057,19 @@
           <bgColor rgb="FFE2F0D9"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2110,29 +2171,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2377,33 +2416,33 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ChangeRegisterTable" displayName="ChangeRegisterTable" ref="A1:Y2" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ChangeRegisterTable" displayName="ChangeRegisterTable" ref="A1:Y4" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47">
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="CHG_ID" dataDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Data" dataDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Título" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Categoria" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Status" dataDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Prioridade" dataDxfId="37"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Responsável" dataDxfId="36"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Fonte/Justificativa" dataDxfId="35"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="REQ_IDs" dataDxfId="34"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ADR_IDs" dataDxfId="33"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Arquivos/paths" dataDxfId="32"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Resumo da alteração" dataDxfId="31"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Razão" dataDxfId="30"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Testes/Gates" dataDxfId="29"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="EVID_IDs" dataDxfId="28"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Branch" dataDxfId="27"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Commit" dataDxfId="26"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="PR" dataDxfId="25"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Release" dataDxfId="24"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Impacto científico" dataDxfId="23"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Impacto numérico" dataDxfId="22"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Impacto API/ABI" dataDxfId="21"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0100-000017000000}" name="Documentação atualizada" dataDxfId="20"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0100-000018000000}" name="Compatibilidade/risco" dataDxfId="19"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0100-000019000000}" name="Observações" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="CHG_ID" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Data" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Título" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Categoria" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Status" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Prioridade" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Responsável" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Fonte/Justificativa" dataDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="REQ_IDs" dataDxfId="41"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ADR_IDs" dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Arquivos/paths" dataDxfId="39"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Resumo da alteração" dataDxfId="38"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Razão" dataDxfId="37"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Testes/Gates" dataDxfId="36"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="EVID_IDs" dataDxfId="35"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Branch" dataDxfId="34"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Commit" dataDxfId="33"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="PR" dataDxfId="32"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Release" dataDxfId="31"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Impacto científico" dataDxfId="30"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Impacto numérico" dataDxfId="29"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Impacto API/ABI" dataDxfId="28"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0100-000017000000}" name="Documentação atualizada" dataDxfId="27"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0100-000018000000}" name="Compatibilidade/risco" dataDxfId="26"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0100-000019000000}" name="Observações" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2434,17 +2473,17 @@
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="RequirementsTable" displayName="RequirementsTable" ref="A1:L60" totalsRowShown="0">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="REQ_ID" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Tipo" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Título" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="REQ_ID" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Tipo" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Título" dataDxfId="22"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Texto normativo"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Estado v0.14" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Fonte" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="ADR_IDs" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="CHG_IDs" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="TEST/Gate_IDs" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="EVID_IDs" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Status implementação" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Estado v0.14" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Fonte" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="ADR_IDs" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="CHG_IDs" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="TEST/Gate_IDs" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="EVID_IDs" dataDxfId="16"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Status implementação" dataDxfId="15"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="Observações"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2456,15 +2495,15 @@
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Record_ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Tipo"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Decisão/Título" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Status" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Fonte" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Decisão/Título" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Status" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Fonte" dataDxfId="12"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="REQ_IDs"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="ADR_file"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Supersedes"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Racional/Evidência"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" name="Responsável"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Data decisão" dataDxfId="45"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Data decisão" dataDxfId="11"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" name="Observações"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6206,13 +6245,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D100">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="10" priority="1">
       <formula>D2="Concluído"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="9" priority="2">
       <formula>D2="Em andamento"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>D2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6237,7 +6276,7 @@
     <col min="3" max="3" width="34" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="6" max="6" width="10" style="26" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="32" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
@@ -6246,7 +6285,7 @@
     <col min="12" max="12" width="48" customWidth="1"/>
     <col min="13" max="13" width="42" customWidth="1"/>
     <col min="14" max="14" width="30" customWidth="1"/>
-    <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="15" max="15" width="27.875" customWidth="1"/>
     <col min="16" max="16" width="24" customWidth="1"/>
     <col min="17" max="17" width="40" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
@@ -6347,9 +6386,9 @@
         <v>150</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="F2" s="8" t="s">
+        <v>564</v>
+      </c>
+      <c r="F2" s="13" t="s">
         <v>72</v>
       </c>
       <c r="G2" s="8" t="s">
@@ -6402,59 +6441,99 @@
         <v>159</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="3"/>
+    <row r="3" spans="1:25" ht="99.75">
+      <c r="A3" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3" s="12">
+        <v>46273</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>581</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>582</v>
+      </c>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="10" t="s">
+        <v>583</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>584</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>585</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>586</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>587</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>588</v>
+      </c>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="8"/>
+      <c r="T3" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="U3" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="V3" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="W3" s="8" t="s">
+        <v>589</v>
+      </c>
+      <c r="X3" s="8" t="s">
+        <v>590</v>
+      </c>
+      <c r="Y3" s="8" t="s">
+        <v>591</v>
+      </c>
     </row>
     <row r="4" spans="1:25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="13"/>
+      <c r="S4" s="8"/>
+      <c r="T4" s="8"/>
+      <c r="U4" s="8"/>
+      <c r="V4" s="8"/>
+      <c r="W4" s="8"/>
+      <c r="X4" s="8"/>
+      <c r="Y4" s="8"/>
     </row>
     <row r="5" spans="1:25">
       <c r="A5" s="3"/>
@@ -6462,7 +6541,7 @@
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="F5" s="5"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -6489,7 +6568,7 @@
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="F6" s="5"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -6516,7 +6595,7 @@
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="F7" s="5"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -6543,7 +6622,7 @@
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="F8" s="5"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -6570,7 +6649,7 @@
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
+      <c r="F9" s="5"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -6597,7 +6676,7 @@
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
+      <c r="F10" s="5"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -6624,7 +6703,7 @@
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
+      <c r="F11" s="5"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -6651,7 +6730,7 @@
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
+      <c r="F12" s="5"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
@@ -6678,7 +6757,7 @@
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
+      <c r="F13" s="5"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -6705,7 +6784,7 @@
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
+      <c r="F14" s="5"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -6732,7 +6811,7 @@
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
+      <c r="F15" s="5"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -6759,7 +6838,7 @@
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
+      <c r="F16" s="5"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
@@ -6786,7 +6865,7 @@
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
+      <c r="F17" s="5"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -6813,7 +6892,7 @@
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
+      <c r="F18" s="5"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -6840,7 +6919,7 @@
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
+      <c r="F19" s="5"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
@@ -6867,7 +6946,7 @@
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
+      <c r="F20" s="5"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
@@ -6894,7 +6973,7 @@
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
+      <c r="F21" s="5"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
@@ -6921,7 +7000,7 @@
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
+      <c r="F22" s="5"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
@@ -6948,7 +7027,7 @@
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="F23" s="5"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
@@ -6975,7 +7054,7 @@
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
+      <c r="F24" s="5"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
@@ -7002,7 +7081,7 @@
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
+      <c r="F25" s="5"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
@@ -7029,7 +7108,7 @@
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
+      <c r="F26" s="5"/>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
@@ -7056,7 +7135,7 @@
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
+      <c r="F27" s="5"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
@@ -7083,7 +7162,7 @@
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
+      <c r="F28" s="5"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -7110,7 +7189,7 @@
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
+      <c r="F29" s="5"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
@@ -7137,7 +7216,7 @@
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
+      <c r="F30" s="5"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
@@ -7164,7 +7243,7 @@
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
+      <c r="F31" s="5"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
@@ -7191,7 +7270,7 @@
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
+      <c r="F32" s="5"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
@@ -7218,7 +7297,7 @@
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
+      <c r="F33" s="5"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
@@ -7245,7 +7324,7 @@
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
+      <c r="F34" s="5"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
@@ -7272,7 +7351,7 @@
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
+      <c r="F35" s="5"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
@@ -7299,7 +7378,7 @@
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
+      <c r="F36" s="5"/>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
@@ -7326,7 +7405,7 @@
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
+      <c r="F37" s="5"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
@@ -7353,7 +7432,7 @@
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
+      <c r="F38" s="5"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
@@ -7380,7 +7459,7 @@
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
+      <c r="F39" s="5"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
@@ -7407,7 +7486,7 @@
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
-      <c r="F40" s="3"/>
+      <c r="F40" s="5"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
@@ -7434,7 +7513,7 @@
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
-      <c r="F41" s="3"/>
+      <c r="F41" s="5"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
@@ -7461,7 +7540,7 @@
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
+      <c r="F42" s="5"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
@@ -7488,7 +7567,7 @@
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
-      <c r="F43" s="3"/>
+      <c r="F43" s="5"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
@@ -7515,7 +7594,7 @@
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
-      <c r="F44" s="3"/>
+      <c r="F44" s="5"/>
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
       <c r="I44" s="3"/>
@@ -7542,7 +7621,7 @@
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
+      <c r="F45" s="5"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
       <c r="I45" s="3"/>
@@ -7569,7 +7648,7 @@
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
+      <c r="F46" s="5"/>
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
       <c r="I46" s="3"/>
@@ -7596,7 +7675,7 @@
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
+      <c r="F47" s="5"/>
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
@@ -7623,7 +7702,7 @@
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
+      <c r="F48" s="5"/>
       <c r="G48" s="3"/>
       <c r="H48" s="3"/>
       <c r="I48" s="3"/>
@@ -7650,7 +7729,7 @@
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
+      <c r="F49" s="5"/>
       <c r="G49" s="3"/>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
@@ -7677,7 +7756,7 @@
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
-      <c r="F50" s="3"/>
+      <c r="F50" s="5"/>
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
       <c r="I50" s="3"/>
@@ -7704,7 +7783,7 @@
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
+      <c r="F51" s="5"/>
       <c r="G51" s="3"/>
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
@@ -7731,7 +7810,7 @@
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
+      <c r="F52" s="5"/>
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
       <c r="I52" s="3"/>
@@ -7758,7 +7837,7 @@
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
+      <c r="F53" s="5"/>
       <c r="G53" s="3"/>
       <c r="H53" s="3"/>
       <c r="I53" s="3"/>
@@ -7785,7 +7864,7 @@
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
+      <c r="F54" s="5"/>
       <c r="G54" s="3"/>
       <c r="H54" s="3"/>
       <c r="I54" s="3"/>
@@ -7812,7 +7891,7 @@
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
-      <c r="F55" s="3"/>
+      <c r="F55" s="5"/>
       <c r="G55" s="3"/>
       <c r="H55" s="3"/>
       <c r="I55" s="3"/>
@@ -7839,7 +7918,7 @@
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
-      <c r="F56" s="3"/>
+      <c r="F56" s="5"/>
       <c r="G56" s="3"/>
       <c r="H56" s="3"/>
       <c r="I56" s="3"/>
@@ -7866,7 +7945,7 @@
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
-      <c r="F57" s="3"/>
+      <c r="F57" s="5"/>
       <c r="G57" s="3"/>
       <c r="H57" s="3"/>
       <c r="I57" s="3"/>
@@ -7893,7 +7972,7 @@
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
+      <c r="F58" s="5"/>
       <c r="G58" s="3"/>
       <c r="H58" s="3"/>
       <c r="I58" s="3"/>
@@ -7920,7 +7999,7 @@
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
+      <c r="F59" s="5"/>
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
       <c r="I59" s="3"/>
@@ -7947,7 +8026,7 @@
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
-      <c r="F60" s="3"/>
+      <c r="F60" s="5"/>
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
       <c r="I60" s="3"/>
@@ -7974,7 +8053,7 @@
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
-      <c r="F61" s="3"/>
+      <c r="F61" s="5"/>
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
       <c r="I61" s="3"/>
@@ -8001,7 +8080,7 @@
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
-      <c r="F62" s="3"/>
+      <c r="F62" s="5"/>
       <c r="G62" s="3"/>
       <c r="H62" s="3"/>
       <c r="I62" s="3"/>
@@ -8028,7 +8107,7 @@
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
       <c r="E63" s="3"/>
-      <c r="F63" s="3"/>
+      <c r="F63" s="5"/>
       <c r="G63" s="3"/>
       <c r="H63" s="3"/>
       <c r="I63" s="3"/>
@@ -8055,7 +8134,7 @@
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
+      <c r="F64" s="5"/>
       <c r="G64" s="3"/>
       <c r="H64" s="3"/>
       <c r="I64" s="3"/>
@@ -8082,7 +8161,7 @@
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
       <c r="E65" s="3"/>
-      <c r="F65" s="3"/>
+      <c r="F65" s="5"/>
       <c r="G65" s="3"/>
       <c r="H65" s="3"/>
       <c r="I65" s="3"/>
@@ -8109,7 +8188,7 @@
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
       <c r="E66" s="3"/>
-      <c r="F66" s="3"/>
+      <c r="F66" s="5"/>
       <c r="G66" s="3"/>
       <c r="H66" s="3"/>
       <c r="I66" s="3"/>
@@ -8136,7 +8215,7 @@
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
       <c r="E67" s="3"/>
-      <c r="F67" s="3"/>
+      <c r="F67" s="5"/>
       <c r="G67" s="3"/>
       <c r="H67" s="3"/>
       <c r="I67" s="3"/>
@@ -8163,7 +8242,7 @@
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
       <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
+      <c r="F68" s="5"/>
       <c r="G68" s="3"/>
       <c r="H68" s="3"/>
       <c r="I68" s="3"/>
@@ -8190,7 +8269,7 @@
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
       <c r="E69" s="3"/>
-      <c r="F69" s="3"/>
+      <c r="F69" s="5"/>
       <c r="G69" s="3"/>
       <c r="H69" s="3"/>
       <c r="I69" s="3"/>
@@ -8217,7 +8296,7 @@
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
-      <c r="F70" s="3"/>
+      <c r="F70" s="5"/>
       <c r="G70" s="3"/>
       <c r="H70" s="3"/>
       <c r="I70" s="3"/>
@@ -8244,7 +8323,7 @@
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
       <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
+      <c r="F71" s="5"/>
       <c r="G71" s="3"/>
       <c r="H71" s="3"/>
       <c r="I71" s="3"/>
@@ -8271,7 +8350,7 @@
       <c r="C72" s="3"/>
       <c r="D72" s="3"/>
       <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
+      <c r="F72" s="5"/>
       <c r="G72" s="3"/>
       <c r="H72" s="3"/>
       <c r="I72" s="3"/>
@@ -8298,7 +8377,7 @@
       <c r="C73" s="3"/>
       <c r="D73" s="3"/>
       <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
+      <c r="F73" s="5"/>
       <c r="G73" s="3"/>
       <c r="H73" s="3"/>
       <c r="I73" s="3"/>
@@ -8325,7 +8404,7 @@
       <c r="C74" s="3"/>
       <c r="D74" s="3"/>
       <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
+      <c r="F74" s="5"/>
       <c r="G74" s="3"/>
       <c r="H74" s="3"/>
       <c r="I74" s="3"/>
@@ -8352,7 +8431,7 @@
       <c r="C75" s="3"/>
       <c r="D75" s="3"/>
       <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
+      <c r="F75" s="5"/>
       <c r="G75" s="3"/>
       <c r="H75" s="3"/>
       <c r="I75" s="3"/>
@@ -8379,7 +8458,7 @@
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
-      <c r="F76" s="3"/>
+      <c r="F76" s="5"/>
       <c r="G76" s="3"/>
       <c r="H76" s="3"/>
       <c r="I76" s="3"/>
@@ -8406,7 +8485,7 @@
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
-      <c r="F77" s="3"/>
+      <c r="F77" s="5"/>
       <c r="G77" s="3"/>
       <c r="H77" s="3"/>
       <c r="I77" s="3"/>
@@ -8433,7 +8512,7 @@
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
-      <c r="F78" s="3"/>
+      <c r="F78" s="5"/>
       <c r="G78" s="3"/>
       <c r="H78" s="3"/>
       <c r="I78" s="3"/>
@@ -8460,7 +8539,7 @@
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
-      <c r="F79" s="3"/>
+      <c r="F79" s="5"/>
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
       <c r="I79" s="3"/>
@@ -8487,7 +8566,7 @@
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
-      <c r="F80" s="3"/>
+      <c r="F80" s="5"/>
       <c r="G80" s="3"/>
       <c r="H80" s="3"/>
       <c r="I80" s="3"/>
@@ -8514,7 +8593,7 @@
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
-      <c r="F81" s="3"/>
+      <c r="F81" s="5"/>
       <c r="G81" s="3"/>
       <c r="H81" s="3"/>
       <c r="I81" s="3"/>
@@ -8541,7 +8620,7 @@
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
-      <c r="F82" s="3"/>
+      <c r="F82" s="5"/>
       <c r="G82" s="3"/>
       <c r="H82" s="3"/>
       <c r="I82" s="3"/>
@@ -8568,7 +8647,7 @@
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
-      <c r="F83" s="3"/>
+      <c r="F83" s="5"/>
       <c r="G83" s="3"/>
       <c r="H83" s="3"/>
       <c r="I83" s="3"/>
@@ -8595,7 +8674,7 @@
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
-      <c r="F84" s="3"/>
+      <c r="F84" s="5"/>
       <c r="G84" s="3"/>
       <c r="H84" s="3"/>
       <c r="I84" s="3"/>
@@ -8622,7 +8701,7 @@
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
-      <c r="F85" s="3"/>
+      <c r="F85" s="5"/>
       <c r="G85" s="3"/>
       <c r="H85" s="3"/>
       <c r="I85" s="3"/>
@@ -8649,7 +8728,7 @@
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
+      <c r="F86" s="5"/>
       <c r="G86" s="3"/>
       <c r="H86" s="3"/>
       <c r="I86" s="3"/>
@@ -8676,7 +8755,7 @@
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
-      <c r="F87" s="3"/>
+      <c r="F87" s="5"/>
       <c r="G87" s="3"/>
       <c r="H87" s="3"/>
       <c r="I87" s="3"/>
@@ -8703,7 +8782,7 @@
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
-      <c r="F88" s="3"/>
+      <c r="F88" s="5"/>
       <c r="G88" s="3"/>
       <c r="H88" s="3"/>
       <c r="I88" s="3"/>
@@ -8730,7 +8809,7 @@
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
-      <c r="F89" s="3"/>
+      <c r="F89" s="5"/>
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
       <c r="I89" s="3"/>
@@ -8757,7 +8836,7 @@
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
-      <c r="F90" s="3"/>
+      <c r="F90" s="5"/>
       <c r="G90" s="3"/>
       <c r="H90" s="3"/>
       <c r="I90" s="3"/>
@@ -8784,7 +8863,7 @@
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
-      <c r="F91" s="3"/>
+      <c r="F91" s="5"/>
       <c r="G91" s="3"/>
       <c r="H91" s="3"/>
       <c r="I91" s="3"/>
@@ -8811,7 +8890,7 @@
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
-      <c r="F92" s="3"/>
+      <c r="F92" s="5"/>
       <c r="G92" s="3"/>
       <c r="H92" s="3"/>
       <c r="I92" s="3"/>
@@ -8838,7 +8917,7 @@
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
-      <c r="F93" s="3"/>
+      <c r="F93" s="5"/>
       <c r="G93" s="3"/>
       <c r="H93" s="3"/>
       <c r="I93" s="3"/>
@@ -8865,7 +8944,7 @@
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
-      <c r="F94" s="3"/>
+      <c r="F94" s="5"/>
       <c r="G94" s="3"/>
       <c r="H94" s="3"/>
       <c r="I94" s="3"/>
@@ -8892,7 +8971,7 @@
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
-      <c r="F95" s="3"/>
+      <c r="F95" s="5"/>
       <c r="G95" s="3"/>
       <c r="H95" s="3"/>
       <c r="I95" s="3"/>
@@ -8919,7 +8998,7 @@
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
-      <c r="F96" s="3"/>
+      <c r="F96" s="5"/>
       <c r="G96" s="3"/>
       <c r="H96" s="3"/>
       <c r="I96" s="3"/>
@@ -8946,7 +9025,7 @@
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
-      <c r="F97" s="3"/>
+      <c r="F97" s="5"/>
       <c r="G97" s="3"/>
       <c r="H97" s="3"/>
       <c r="I97" s="3"/>
@@ -8973,7 +9052,7 @@
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
-      <c r="F98" s="3"/>
+      <c r="F98" s="5"/>
       <c r="G98" s="3"/>
       <c r="H98" s="3"/>
       <c r="I98" s="3"/>
@@ -9000,7 +9079,7 @@
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
-      <c r="F99" s="3"/>
+      <c r="F99" s="5"/>
       <c r="G99" s="3"/>
       <c r="H99" s="3"/>
       <c r="I99" s="3"/>
@@ -9027,7 +9106,7 @@
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
-      <c r="F100" s="3"/>
+      <c r="F100" s="5"/>
       <c r="G100" s="3"/>
       <c r="H100" s="3"/>
       <c r="I100" s="3"/>
@@ -9054,7 +9133,7 @@
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>
       <c r="E101" s="3"/>
-      <c r="F101" s="3"/>
+      <c r="F101" s="5"/>
       <c r="G101" s="3"/>
       <c r="H101" s="3"/>
       <c r="I101" s="3"/>
@@ -9081,7 +9160,7 @@
       <c r="C102" s="3"/>
       <c r="D102" s="3"/>
       <c r="E102" s="3"/>
-      <c r="F102" s="3"/>
+      <c r="F102" s="5"/>
       <c r="G102" s="3"/>
       <c r="H102" s="3"/>
       <c r="I102" s="3"/>
@@ -9108,7 +9187,7 @@
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
       <c r="E103" s="3"/>
-      <c r="F103" s="3"/>
+      <c r="F103" s="5"/>
       <c r="G103" s="3"/>
       <c r="H103" s="3"/>
       <c r="I103" s="3"/>
@@ -9135,7 +9214,7 @@
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
-      <c r="F104" s="3"/>
+      <c r="F104" s="5"/>
       <c r="G104" s="3"/>
       <c r="H104" s="3"/>
       <c r="I104" s="3"/>
@@ -9162,7 +9241,7 @@
       <c r="C105" s="3"/>
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
-      <c r="F105" s="3"/>
+      <c r="F105" s="5"/>
       <c r="G105" s="3"/>
       <c r="H105" s="3"/>
       <c r="I105" s="3"/>
@@ -9189,7 +9268,7 @@
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
-      <c r="F106" s="3"/>
+      <c r="F106" s="5"/>
       <c r="G106" s="3"/>
       <c r="H106" s="3"/>
       <c r="I106" s="3"/>
@@ -9216,7 +9295,7 @@
       <c r="C107" s="3"/>
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
-      <c r="F107" s="3"/>
+      <c r="F107" s="5"/>
       <c r="G107" s="3"/>
       <c r="H107" s="3"/>
       <c r="I107" s="3"/>
@@ -9243,7 +9322,7 @@
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
-      <c r="F108" s="3"/>
+      <c r="F108" s="5"/>
       <c r="G108" s="3"/>
       <c r="H108" s="3"/>
       <c r="I108" s="3"/>
@@ -9270,7 +9349,7 @@
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
       <c r="E109" s="3"/>
-      <c r="F109" s="3"/>
+      <c r="F109" s="5"/>
       <c r="G109" s="3"/>
       <c r="H109" s="3"/>
       <c r="I109" s="3"/>
@@ -9297,7 +9376,7 @@
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
-      <c r="F110" s="3"/>
+      <c r="F110" s="5"/>
       <c r="G110" s="3"/>
       <c r="H110" s="3"/>
       <c r="I110" s="3"/>
@@ -9324,7 +9403,7 @@
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
       <c r="E111" s="3"/>
-      <c r="F111" s="3"/>
+      <c r="F111" s="5"/>
       <c r="G111" s="3"/>
       <c r="H111" s="3"/>
       <c r="I111" s="3"/>
@@ -9351,7 +9430,7 @@
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
-      <c r="F112" s="3"/>
+      <c r="F112" s="5"/>
       <c r="G112" s="3"/>
       <c r="H112" s="3"/>
       <c r="I112" s="3"/>
@@ -9378,7 +9457,7 @@
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
       <c r="E113" s="3"/>
-      <c r="F113" s="3"/>
+      <c r="F113" s="5"/>
       <c r="G113" s="3"/>
       <c r="H113" s="3"/>
       <c r="I113" s="3"/>
@@ -9405,7 +9484,7 @@
       <c r="C114" s="3"/>
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
-      <c r="F114" s="3"/>
+      <c r="F114" s="5"/>
       <c r="G114" s="3"/>
       <c r="H114" s="3"/>
       <c r="I114" s="3"/>
@@ -9432,7 +9511,7 @@
       <c r="C115" s="3"/>
       <c r="D115" s="3"/>
       <c r="E115" s="3"/>
-      <c r="F115" s="3"/>
+      <c r="F115" s="5"/>
       <c r="G115" s="3"/>
       <c r="H115" s="3"/>
       <c r="I115" s="3"/>
@@ -9459,7 +9538,7 @@
       <c r="C116" s="3"/>
       <c r="D116" s="3"/>
       <c r="E116" s="3"/>
-      <c r="F116" s="3"/>
+      <c r="F116" s="5"/>
       <c r="G116" s="3"/>
       <c r="H116" s="3"/>
       <c r="I116" s="3"/>
@@ -9486,7 +9565,7 @@
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
       <c r="E117" s="3"/>
-      <c r="F117" s="3"/>
+      <c r="F117" s="5"/>
       <c r="G117" s="3"/>
       <c r="H117" s="3"/>
       <c r="I117" s="3"/>
@@ -9513,7 +9592,7 @@
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
       <c r="E118" s="3"/>
-      <c r="F118" s="3"/>
+      <c r="F118" s="5"/>
       <c r="G118" s="3"/>
       <c r="H118" s="3"/>
       <c r="I118" s="3"/>
@@ -9540,7 +9619,7 @@
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
       <c r="E119" s="3"/>
-      <c r="F119" s="3"/>
+      <c r="F119" s="5"/>
       <c r="G119" s="3"/>
       <c r="H119" s="3"/>
       <c r="I119" s="3"/>
@@ -9567,7 +9646,7 @@
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
       <c r="E120" s="3"/>
-      <c r="F120" s="3"/>
+      <c r="F120" s="5"/>
       <c r="G120" s="3"/>
       <c r="H120" s="3"/>
       <c r="I120" s="3"/>
@@ -9594,7 +9673,7 @@
       <c r="C121" s="3"/>
       <c r="D121" s="3"/>
       <c r="E121" s="3"/>
-      <c r="F121" s="3"/>
+      <c r="F121" s="5"/>
       <c r="G121" s="3"/>
       <c r="H121" s="3"/>
       <c r="I121" s="3"/>
@@ -9621,7 +9700,7 @@
       <c r="C122" s="3"/>
       <c r="D122" s="3"/>
       <c r="E122" s="3"/>
-      <c r="F122" s="3"/>
+      <c r="F122" s="5"/>
       <c r="G122" s="3"/>
       <c r="H122" s="3"/>
       <c r="I122" s="3"/>
@@ -9648,7 +9727,7 @@
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
       <c r="E123" s="3"/>
-      <c r="F123" s="3"/>
+      <c r="F123" s="5"/>
       <c r="G123" s="3"/>
       <c r="H123" s="3"/>
       <c r="I123" s="3"/>
@@ -9675,7 +9754,7 @@
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
       <c r="E124" s="3"/>
-      <c r="F124" s="3"/>
+      <c r="F124" s="5"/>
       <c r="G124" s="3"/>
       <c r="H124" s="3"/>
       <c r="I124" s="3"/>
@@ -9702,7 +9781,7 @@
       <c r="C125" s="3"/>
       <c r="D125" s="3"/>
       <c r="E125" s="3"/>
-      <c r="F125" s="3"/>
+      <c r="F125" s="5"/>
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
       <c r="I125" s="3"/>
@@ -9729,7 +9808,7 @@
       <c r="C126" s="3"/>
       <c r="D126" s="3"/>
       <c r="E126" s="3"/>
-      <c r="F126" s="3"/>
+      <c r="F126" s="5"/>
       <c r="G126" s="3"/>
       <c r="H126" s="3"/>
       <c r="I126" s="3"/>
@@ -9756,7 +9835,7 @@
       <c r="C127" s="3"/>
       <c r="D127" s="3"/>
       <c r="E127" s="3"/>
-      <c r="F127" s="3"/>
+      <c r="F127" s="5"/>
       <c r="G127" s="3"/>
       <c r="H127" s="3"/>
       <c r="I127" s="3"/>
@@ -9783,7 +9862,7 @@
       <c r="C128" s="3"/>
       <c r="D128" s="3"/>
       <c r="E128" s="3"/>
-      <c r="F128" s="3"/>
+      <c r="F128" s="5"/>
       <c r="G128" s="3"/>
       <c r="H128" s="3"/>
       <c r="I128" s="3"/>
@@ -9810,7 +9889,7 @@
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
       <c r="E129" s="3"/>
-      <c r="F129" s="3"/>
+      <c r="F129" s="5"/>
       <c r="G129" s="3"/>
       <c r="H129" s="3"/>
       <c r="I129" s="3"/>
@@ -9837,7 +9916,7 @@
       <c r="C130" s="3"/>
       <c r="D130" s="3"/>
       <c r="E130" s="3"/>
-      <c r="F130" s="3"/>
+      <c r="F130" s="5"/>
       <c r="G130" s="3"/>
       <c r="H130" s="3"/>
       <c r="I130" s="3"/>
@@ -9864,7 +9943,7 @@
       <c r="C131" s="3"/>
       <c r="D131" s="3"/>
       <c r="E131" s="3"/>
-      <c r="F131" s="3"/>
+      <c r="F131" s="5"/>
       <c r="G131" s="3"/>
       <c r="H131" s="3"/>
       <c r="I131" s="3"/>
@@ -9891,7 +9970,7 @@
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
       <c r="E132" s="3"/>
-      <c r="F132" s="3"/>
+      <c r="F132" s="5"/>
       <c r="G132" s="3"/>
       <c r="H132" s="3"/>
       <c r="I132" s="3"/>
@@ -9918,7 +9997,7 @@
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
       <c r="E133" s="3"/>
-      <c r="F133" s="3"/>
+      <c r="F133" s="5"/>
       <c r="G133" s="3"/>
       <c r="H133" s="3"/>
       <c r="I133" s="3"/>
@@ -9945,7 +10024,7 @@
       <c r="C134" s="3"/>
       <c r="D134" s="3"/>
       <c r="E134" s="3"/>
-      <c r="F134" s="3"/>
+      <c r="F134" s="5"/>
       <c r="G134" s="3"/>
       <c r="H134" s="3"/>
       <c r="I134" s="3"/>
@@ -9972,7 +10051,7 @@
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
       <c r="E135" s="3"/>
-      <c r="F135" s="3"/>
+      <c r="F135" s="5"/>
       <c r="G135" s="3"/>
       <c r="H135" s="3"/>
       <c r="I135" s="3"/>
@@ -9999,7 +10078,7 @@
       <c r="C136" s="3"/>
       <c r="D136" s="3"/>
       <c r="E136" s="3"/>
-      <c r="F136" s="3"/>
+      <c r="F136" s="5"/>
       <c r="G136" s="3"/>
       <c r="H136" s="3"/>
       <c r="I136" s="3"/>
@@ -10026,7 +10105,7 @@
       <c r="C137" s="3"/>
       <c r="D137" s="3"/>
       <c r="E137" s="3"/>
-      <c r="F137" s="3"/>
+      <c r="F137" s="5"/>
       <c r="G137" s="3"/>
       <c r="H137" s="3"/>
       <c r="I137" s="3"/>
@@ -10053,7 +10132,7 @@
       <c r="C138" s="3"/>
       <c r="D138" s="3"/>
       <c r="E138" s="3"/>
-      <c r="F138" s="3"/>
+      <c r="F138" s="5"/>
       <c r="G138" s="3"/>
       <c r="H138" s="3"/>
       <c r="I138" s="3"/>
@@ -10080,7 +10159,7 @@
       <c r="C139" s="3"/>
       <c r="D139" s="3"/>
       <c r="E139" s="3"/>
-      <c r="F139" s="3"/>
+      <c r="F139" s="5"/>
       <c r="G139" s="3"/>
       <c r="H139" s="3"/>
       <c r="I139" s="3"/>
@@ -10107,7 +10186,7 @@
       <c r="C140" s="3"/>
       <c r="D140" s="3"/>
       <c r="E140" s="3"/>
-      <c r="F140" s="3"/>
+      <c r="F140" s="5"/>
       <c r="G140" s="3"/>
       <c r="H140" s="3"/>
       <c r="I140" s="3"/>
@@ -10134,7 +10213,7 @@
       <c r="C141" s="3"/>
       <c r="D141" s="3"/>
       <c r="E141" s="3"/>
-      <c r="F141" s="3"/>
+      <c r="F141" s="5"/>
       <c r="G141" s="3"/>
       <c r="H141" s="3"/>
       <c r="I141" s="3"/>
@@ -10161,7 +10240,7 @@
       <c r="C142" s="3"/>
       <c r="D142" s="3"/>
       <c r="E142" s="3"/>
-      <c r="F142" s="3"/>
+      <c r="F142" s="5"/>
       <c r="G142" s="3"/>
       <c r="H142" s="3"/>
       <c r="I142" s="3"/>
@@ -10188,7 +10267,7 @@
       <c r="C143" s="3"/>
       <c r="D143" s="3"/>
       <c r="E143" s="3"/>
-      <c r="F143" s="3"/>
+      <c r="F143" s="5"/>
       <c r="G143" s="3"/>
       <c r="H143" s="3"/>
       <c r="I143" s="3"/>
@@ -10215,7 +10294,7 @@
       <c r="C144" s="3"/>
       <c r="D144" s="3"/>
       <c r="E144" s="3"/>
-      <c r="F144" s="3"/>
+      <c r="F144" s="5"/>
       <c r="G144" s="3"/>
       <c r="H144" s="3"/>
       <c r="I144" s="3"/>
@@ -10242,7 +10321,7 @@
       <c r="C145" s="3"/>
       <c r="D145" s="3"/>
       <c r="E145" s="3"/>
-      <c r="F145" s="3"/>
+      <c r="F145" s="5"/>
       <c r="G145" s="3"/>
       <c r="H145" s="3"/>
       <c r="I145" s="3"/>
@@ -10269,7 +10348,7 @@
       <c r="C146" s="3"/>
       <c r="D146" s="3"/>
       <c r="E146" s="3"/>
-      <c r="F146" s="3"/>
+      <c r="F146" s="5"/>
       <c r="G146" s="3"/>
       <c r="H146" s="3"/>
       <c r="I146" s="3"/>
@@ -10296,7 +10375,7 @@
       <c r="C147" s="3"/>
       <c r="D147" s="3"/>
       <c r="E147" s="3"/>
-      <c r="F147" s="3"/>
+      <c r="F147" s="5"/>
       <c r="G147" s="3"/>
       <c r="H147" s="3"/>
       <c r="I147" s="3"/>
@@ -10323,7 +10402,7 @@
       <c r="C148" s="3"/>
       <c r="D148" s="3"/>
       <c r="E148" s="3"/>
-      <c r="F148" s="3"/>
+      <c r="F148" s="5"/>
       <c r="G148" s="3"/>
       <c r="H148" s="3"/>
       <c r="I148" s="3"/>
@@ -10350,7 +10429,7 @@
       <c r="C149" s="3"/>
       <c r="D149" s="3"/>
       <c r="E149" s="3"/>
-      <c r="F149" s="3"/>
+      <c r="F149" s="5"/>
       <c r="G149" s="3"/>
       <c r="H149" s="3"/>
       <c r="I149" s="3"/>
@@ -10377,7 +10456,7 @@
       <c r="C150" s="3"/>
       <c r="D150" s="3"/>
       <c r="E150" s="3"/>
-      <c r="F150" s="3"/>
+      <c r="F150" s="5"/>
       <c r="G150" s="3"/>
       <c r="H150" s="3"/>
       <c r="I150" s="3"/>
@@ -10404,7 +10483,7 @@
       <c r="C151" s="3"/>
       <c r="D151" s="3"/>
       <c r="E151" s="3"/>
-      <c r="F151" s="3"/>
+      <c r="F151" s="5"/>
       <c r="G151" s="3"/>
       <c r="H151" s="3"/>
       <c r="I151" s="3"/>
@@ -10431,7 +10510,7 @@
       <c r="C152" s="3"/>
       <c r="D152" s="3"/>
       <c r="E152" s="3"/>
-      <c r="F152" s="3"/>
+      <c r="F152" s="5"/>
       <c r="G152" s="3"/>
       <c r="H152" s="3"/>
       <c r="I152" s="3"/>
@@ -10458,7 +10537,7 @@
       <c r="C153" s="3"/>
       <c r="D153" s="3"/>
       <c r="E153" s="3"/>
-      <c r="F153" s="3"/>
+      <c r="F153" s="5"/>
       <c r="G153" s="3"/>
       <c r="H153" s="3"/>
       <c r="I153" s="3"/>
@@ -10485,7 +10564,7 @@
       <c r="C154" s="3"/>
       <c r="D154" s="3"/>
       <c r="E154" s="3"/>
-      <c r="F154" s="3"/>
+      <c r="F154" s="5"/>
       <c r="G154" s="3"/>
       <c r="H154" s="3"/>
       <c r="I154" s="3"/>
@@ -10512,7 +10591,7 @@
       <c r="C155" s="3"/>
       <c r="D155" s="3"/>
       <c r="E155" s="3"/>
-      <c r="F155" s="3"/>
+      <c r="F155" s="5"/>
       <c r="G155" s="3"/>
       <c r="H155" s="3"/>
       <c r="I155" s="3"/>
@@ -10539,7 +10618,7 @@
       <c r="C156" s="3"/>
       <c r="D156" s="3"/>
       <c r="E156" s="3"/>
-      <c r="F156" s="3"/>
+      <c r="F156" s="5"/>
       <c r="G156" s="3"/>
       <c r="H156" s="3"/>
       <c r="I156" s="3"/>
@@ -10566,7 +10645,7 @@
       <c r="C157" s="3"/>
       <c r="D157" s="3"/>
       <c r="E157" s="3"/>
-      <c r="F157" s="3"/>
+      <c r="F157" s="5"/>
       <c r="G157" s="3"/>
       <c r="H157" s="3"/>
       <c r="I157" s="3"/>
@@ -10593,7 +10672,7 @@
       <c r="C158" s="3"/>
       <c r="D158" s="3"/>
       <c r="E158" s="3"/>
-      <c r="F158" s="3"/>
+      <c r="F158" s="5"/>
       <c r="G158" s="3"/>
       <c r="H158" s="3"/>
       <c r="I158" s="3"/>
@@ -10620,7 +10699,7 @@
       <c r="C159" s="3"/>
       <c r="D159" s="3"/>
       <c r="E159" s="3"/>
-      <c r="F159" s="3"/>
+      <c r="F159" s="5"/>
       <c r="G159" s="3"/>
       <c r="H159" s="3"/>
       <c r="I159" s="3"/>
@@ -10647,7 +10726,7 @@
       <c r="C160" s="3"/>
       <c r="D160" s="3"/>
       <c r="E160" s="3"/>
-      <c r="F160" s="3"/>
+      <c r="F160" s="5"/>
       <c r="G160" s="3"/>
       <c r="H160" s="3"/>
       <c r="I160" s="3"/>
@@ -10674,7 +10753,7 @@
       <c r="C161" s="3"/>
       <c r="D161" s="3"/>
       <c r="E161" s="3"/>
-      <c r="F161" s="3"/>
+      <c r="F161" s="5"/>
       <c r="G161" s="3"/>
       <c r="H161" s="3"/>
       <c r="I161" s="3"/>
@@ -10701,7 +10780,7 @@
       <c r="C162" s="3"/>
       <c r="D162" s="3"/>
       <c r="E162" s="3"/>
-      <c r="F162" s="3"/>
+      <c r="F162" s="5"/>
       <c r="G162" s="3"/>
       <c r="H162" s="3"/>
       <c r="I162" s="3"/>
@@ -10728,7 +10807,7 @@
       <c r="C163" s="3"/>
       <c r="D163" s="3"/>
       <c r="E163" s="3"/>
-      <c r="F163" s="3"/>
+      <c r="F163" s="5"/>
       <c r="G163" s="3"/>
       <c r="H163" s="3"/>
       <c r="I163" s="3"/>
@@ -10755,7 +10834,7 @@
       <c r="C164" s="3"/>
       <c r="D164" s="3"/>
       <c r="E164" s="3"/>
-      <c r="F164" s="3"/>
+      <c r="F164" s="5"/>
       <c r="G164" s="3"/>
       <c r="H164" s="3"/>
       <c r="I164" s="3"/>
@@ -10782,7 +10861,7 @@
       <c r="C165" s="3"/>
       <c r="D165" s="3"/>
       <c r="E165" s="3"/>
-      <c r="F165" s="3"/>
+      <c r="F165" s="5"/>
       <c r="G165" s="3"/>
       <c r="H165" s="3"/>
       <c r="I165" s="3"/>
@@ -10809,7 +10888,7 @@
       <c r="C166" s="3"/>
       <c r="D166" s="3"/>
       <c r="E166" s="3"/>
-      <c r="F166" s="3"/>
+      <c r="F166" s="5"/>
       <c r="G166" s="3"/>
       <c r="H166" s="3"/>
       <c r="I166" s="3"/>
@@ -10836,7 +10915,7 @@
       <c r="C167" s="3"/>
       <c r="D167" s="3"/>
       <c r="E167" s="3"/>
-      <c r="F167" s="3"/>
+      <c r="F167" s="5"/>
       <c r="G167" s="3"/>
       <c r="H167" s="3"/>
       <c r="I167" s="3"/>
@@ -10863,7 +10942,7 @@
       <c r="C168" s="3"/>
       <c r="D168" s="3"/>
       <c r="E168" s="3"/>
-      <c r="F168" s="3"/>
+      <c r="F168" s="5"/>
       <c r="G168" s="3"/>
       <c r="H168" s="3"/>
       <c r="I168" s="3"/>
@@ -10890,7 +10969,7 @@
       <c r="C169" s="3"/>
       <c r="D169" s="3"/>
       <c r="E169" s="3"/>
-      <c r="F169" s="3"/>
+      <c r="F169" s="5"/>
       <c r="G169" s="3"/>
       <c r="H169" s="3"/>
       <c r="I169" s="3"/>
@@ -10917,7 +10996,7 @@
       <c r="C170" s="3"/>
       <c r="D170" s="3"/>
       <c r="E170" s="3"/>
-      <c r="F170" s="3"/>
+      <c r="F170" s="5"/>
       <c r="G170" s="3"/>
       <c r="H170" s="3"/>
       <c r="I170" s="3"/>
@@ -10944,7 +11023,7 @@
       <c r="C171" s="3"/>
       <c r="D171" s="3"/>
       <c r="E171" s="3"/>
-      <c r="F171" s="3"/>
+      <c r="F171" s="5"/>
       <c r="G171" s="3"/>
       <c r="H171" s="3"/>
       <c r="I171" s="3"/>
@@ -10971,7 +11050,7 @@
       <c r="C172" s="3"/>
       <c r="D172" s="3"/>
       <c r="E172" s="3"/>
-      <c r="F172" s="3"/>
+      <c r="F172" s="5"/>
       <c r="G172" s="3"/>
       <c r="H172" s="3"/>
       <c r="I172" s="3"/>
@@ -10998,7 +11077,7 @@
       <c r="C173" s="3"/>
       <c r="D173" s="3"/>
       <c r="E173" s="3"/>
-      <c r="F173" s="3"/>
+      <c r="F173" s="5"/>
       <c r="G173" s="3"/>
       <c r="H173" s="3"/>
       <c r="I173" s="3"/>
@@ -11025,7 +11104,7 @@
       <c r="C174" s="3"/>
       <c r="D174" s="3"/>
       <c r="E174" s="3"/>
-      <c r="F174" s="3"/>
+      <c r="F174" s="5"/>
       <c r="G174" s="3"/>
       <c r="H174" s="3"/>
       <c r="I174" s="3"/>
@@ -11052,7 +11131,7 @@
       <c r="C175" s="3"/>
       <c r="D175" s="3"/>
       <c r="E175" s="3"/>
-      <c r="F175" s="3"/>
+      <c r="F175" s="5"/>
       <c r="G175" s="3"/>
       <c r="H175" s="3"/>
       <c r="I175" s="3"/>
@@ -11079,7 +11158,7 @@
       <c r="C176" s="3"/>
       <c r="D176" s="3"/>
       <c r="E176" s="3"/>
-      <c r="F176" s="3"/>
+      <c r="F176" s="5"/>
       <c r="G176" s="3"/>
       <c r="H176" s="3"/>
       <c r="I176" s="3"/>
@@ -11106,7 +11185,7 @@
       <c r="C177" s="3"/>
       <c r="D177" s="3"/>
       <c r="E177" s="3"/>
-      <c r="F177" s="3"/>
+      <c r="F177" s="5"/>
       <c r="G177" s="3"/>
       <c r="H177" s="3"/>
       <c r="I177" s="3"/>
@@ -11133,7 +11212,7 @@
       <c r="C178" s="3"/>
       <c r="D178" s="3"/>
       <c r="E178" s="3"/>
-      <c r="F178" s="3"/>
+      <c r="F178" s="5"/>
       <c r="G178" s="3"/>
       <c r="H178" s="3"/>
       <c r="I178" s="3"/>
@@ -11160,7 +11239,7 @@
       <c r="C179" s="3"/>
       <c r="D179" s="3"/>
       <c r="E179" s="3"/>
-      <c r="F179" s="3"/>
+      <c r="F179" s="5"/>
       <c r="G179" s="3"/>
       <c r="H179" s="3"/>
       <c r="I179" s="3"/>
@@ -11187,7 +11266,7 @@
       <c r="C180" s="3"/>
       <c r="D180" s="3"/>
       <c r="E180" s="3"/>
-      <c r="F180" s="3"/>
+      <c r="F180" s="5"/>
       <c r="G180" s="3"/>
       <c r="H180" s="3"/>
       <c r="I180" s="3"/>
@@ -11214,7 +11293,7 @@
       <c r="C181" s="3"/>
       <c r="D181" s="3"/>
       <c r="E181" s="3"/>
-      <c r="F181" s="3"/>
+      <c r="F181" s="5"/>
       <c r="G181" s="3"/>
       <c r="H181" s="3"/>
       <c r="I181" s="3"/>
@@ -11241,7 +11320,7 @@
       <c r="C182" s="3"/>
       <c r="D182" s="3"/>
       <c r="E182" s="3"/>
-      <c r="F182" s="3"/>
+      <c r="F182" s="5"/>
       <c r="G182" s="3"/>
       <c r="H182" s="3"/>
       <c r="I182" s="3"/>
@@ -11268,7 +11347,7 @@
       <c r="C183" s="3"/>
       <c r="D183" s="3"/>
       <c r="E183" s="3"/>
-      <c r="F183" s="3"/>
+      <c r="F183" s="5"/>
       <c r="G183" s="3"/>
       <c r="H183" s="3"/>
       <c r="I183" s="3"/>
@@ -11295,7 +11374,7 @@
       <c r="C184" s="3"/>
       <c r="D184" s="3"/>
       <c r="E184" s="3"/>
-      <c r="F184" s="3"/>
+      <c r="F184" s="5"/>
       <c r="G184" s="3"/>
       <c r="H184" s="3"/>
       <c r="I184" s="3"/>
@@ -11322,7 +11401,7 @@
       <c r="C185" s="3"/>
       <c r="D185" s="3"/>
       <c r="E185" s="3"/>
-      <c r="F185" s="3"/>
+      <c r="F185" s="5"/>
       <c r="G185" s="3"/>
       <c r="H185" s="3"/>
       <c r="I185" s="3"/>
@@ -11349,7 +11428,7 @@
       <c r="C186" s="3"/>
       <c r="D186" s="3"/>
       <c r="E186" s="3"/>
-      <c r="F186" s="3"/>
+      <c r="F186" s="5"/>
       <c r="G186" s="3"/>
       <c r="H186" s="3"/>
       <c r="I186" s="3"/>
@@ -11376,7 +11455,7 @@
       <c r="C187" s="3"/>
       <c r="D187" s="3"/>
       <c r="E187" s="3"/>
-      <c r="F187" s="3"/>
+      <c r="F187" s="5"/>
       <c r="G187" s="3"/>
       <c r="H187" s="3"/>
       <c r="I187" s="3"/>
@@ -11403,7 +11482,7 @@
       <c r="C188" s="3"/>
       <c r="D188" s="3"/>
       <c r="E188" s="3"/>
-      <c r="F188" s="3"/>
+      <c r="F188" s="5"/>
       <c r="G188" s="3"/>
       <c r="H188" s="3"/>
       <c r="I188" s="3"/>
@@ -11430,7 +11509,7 @@
       <c r="C189" s="3"/>
       <c r="D189" s="3"/>
       <c r="E189" s="3"/>
-      <c r="F189" s="3"/>
+      <c r="F189" s="5"/>
       <c r="G189" s="3"/>
       <c r="H189" s="3"/>
       <c r="I189" s="3"/>
@@ -11457,7 +11536,7 @@
       <c r="C190" s="3"/>
       <c r="D190" s="3"/>
       <c r="E190" s="3"/>
-      <c r="F190" s="3"/>
+      <c r="F190" s="5"/>
       <c r="G190" s="3"/>
       <c r="H190" s="3"/>
       <c r="I190" s="3"/>
@@ -11484,7 +11563,7 @@
       <c r="C191" s="3"/>
       <c r="D191" s="3"/>
       <c r="E191" s="3"/>
-      <c r="F191" s="3"/>
+      <c r="F191" s="5"/>
       <c r="G191" s="3"/>
       <c r="H191" s="3"/>
       <c r="I191" s="3"/>
@@ -11511,7 +11590,7 @@
       <c r="C192" s="3"/>
       <c r="D192" s="3"/>
       <c r="E192" s="3"/>
-      <c r="F192" s="3"/>
+      <c r="F192" s="5"/>
       <c r="G192" s="3"/>
       <c r="H192" s="3"/>
       <c r="I192" s="3"/>
@@ -11538,7 +11617,7 @@
       <c r="C193" s="3"/>
       <c r="D193" s="3"/>
       <c r="E193" s="3"/>
-      <c r="F193" s="3"/>
+      <c r="F193" s="5"/>
       <c r="G193" s="3"/>
       <c r="H193" s="3"/>
       <c r="I193" s="3"/>
@@ -11565,7 +11644,7 @@
       <c r="C194" s="3"/>
       <c r="D194" s="3"/>
       <c r="E194" s="3"/>
-      <c r="F194" s="3"/>
+      <c r="F194" s="5"/>
       <c r="G194" s="3"/>
       <c r="H194" s="3"/>
       <c r="I194" s="3"/>
@@ -11592,7 +11671,7 @@
       <c r="C195" s="3"/>
       <c r="D195" s="3"/>
       <c r="E195" s="3"/>
-      <c r="F195" s="3"/>
+      <c r="F195" s="5"/>
       <c r="G195" s="3"/>
       <c r="H195" s="3"/>
       <c r="I195" s="3"/>
@@ -11619,7 +11698,7 @@
       <c r="C196" s="3"/>
       <c r="D196" s="3"/>
       <c r="E196" s="3"/>
-      <c r="F196" s="3"/>
+      <c r="F196" s="5"/>
       <c r="G196" s="3"/>
       <c r="H196" s="3"/>
       <c r="I196" s="3"/>
@@ -11646,7 +11725,7 @@
       <c r="C197" s="3"/>
       <c r="D197" s="3"/>
       <c r="E197" s="3"/>
-      <c r="F197" s="3"/>
+      <c r="F197" s="5"/>
       <c r="G197" s="3"/>
       <c r="H197" s="3"/>
       <c r="I197" s="3"/>
@@ -11673,7 +11752,7 @@
       <c r="C198" s="3"/>
       <c r="D198" s="3"/>
       <c r="E198" s="3"/>
-      <c r="F198" s="3"/>
+      <c r="F198" s="5"/>
       <c r="G198" s="3"/>
       <c r="H198" s="3"/>
       <c r="I198" s="3"/>
@@ -11700,7 +11779,7 @@
       <c r="C199" s="3"/>
       <c r="D199" s="3"/>
       <c r="E199" s="3"/>
-      <c r="F199" s="3"/>
+      <c r="F199" s="5"/>
       <c r="G199" s="3"/>
       <c r="H199" s="3"/>
       <c r="I199" s="3"/>
@@ -11727,7 +11806,7 @@
       <c r="C200" s="3"/>
       <c r="D200" s="3"/>
       <c r="E200" s="3"/>
-      <c r="F200" s="3"/>
+      <c r="F200" s="5"/>
       <c r="G200" s="3"/>
       <c r="H200" s="3"/>
       <c r="I200" s="3"/>
@@ -11754,7 +11833,7 @@
       <c r="C201" s="3"/>
       <c r="D201" s="3"/>
       <c r="E201" s="3"/>
-      <c r="F201" s="3"/>
+      <c r="F201" s="5"/>
       <c r="G201" s="3"/>
       <c r="H201" s="3"/>
       <c r="I201" s="3"/>
@@ -11781,7 +11860,7 @@
       <c r="C202" s="3"/>
       <c r="D202" s="3"/>
       <c r="E202" s="3"/>
-      <c r="F202" s="3"/>
+      <c r="F202" s="5"/>
       <c r="G202" s="3"/>
       <c r="H202" s="3"/>
       <c r="I202" s="3"/>
@@ -11808,7 +11887,7 @@
       <c r="C203" s="3"/>
       <c r="D203" s="3"/>
       <c r="E203" s="3"/>
-      <c r="F203" s="3"/>
+      <c r="F203" s="5"/>
       <c r="G203" s="3"/>
       <c r="H203" s="3"/>
       <c r="I203" s="3"/>
@@ -11835,7 +11914,7 @@
       <c r="C204" s="3"/>
       <c r="D204" s="3"/>
       <c r="E204" s="3"/>
-      <c r="F204" s="3"/>
+      <c r="F204" s="5"/>
       <c r="G204" s="3"/>
       <c r="H204" s="3"/>
       <c r="I204" s="3"/>
@@ -11862,7 +11941,7 @@
       <c r="C205" s="3"/>
       <c r="D205" s="3"/>
       <c r="E205" s="3"/>
-      <c r="F205" s="3"/>
+      <c r="F205" s="5"/>
       <c r="G205" s="3"/>
       <c r="H205" s="3"/>
       <c r="I205" s="3"/>
@@ -11889,7 +11968,7 @@
       <c r="C206" s="3"/>
       <c r="D206" s="3"/>
       <c r="E206" s="3"/>
-      <c r="F206" s="3"/>
+      <c r="F206" s="5"/>
       <c r="G206" s="3"/>
       <c r="H206" s="3"/>
       <c r="I206" s="3"/>
@@ -11916,7 +11995,7 @@
       <c r="C207" s="3"/>
       <c r="D207" s="3"/>
       <c r="E207" s="3"/>
-      <c r="F207" s="3"/>
+      <c r="F207" s="5"/>
       <c r="G207" s="3"/>
       <c r="H207" s="3"/>
       <c r="I207" s="3"/>
@@ -11943,7 +12022,7 @@
       <c r="C208" s="3"/>
       <c r="D208" s="3"/>
       <c r="E208" s="3"/>
-      <c r="F208" s="3"/>
+      <c r="F208" s="5"/>
       <c r="G208" s="3"/>
       <c r="H208" s="3"/>
       <c r="I208" s="3"/>
@@ -11970,7 +12049,7 @@
       <c r="C209" s="3"/>
       <c r="D209" s="3"/>
       <c r="E209" s="3"/>
-      <c r="F209" s="3"/>
+      <c r="F209" s="5"/>
       <c r="G209" s="3"/>
       <c r="H209" s="3"/>
       <c r="I209" s="3"/>
@@ -11997,7 +12076,7 @@
       <c r="C210" s="3"/>
       <c r="D210" s="3"/>
       <c r="E210" s="3"/>
-      <c r="F210" s="3"/>
+      <c r="F210" s="5"/>
       <c r="G210" s="3"/>
       <c r="H210" s="3"/>
       <c r="I210" s="3"/>
@@ -12024,7 +12103,7 @@
       <c r="C211" s="3"/>
       <c r="D211" s="3"/>
       <c r="E211" s="3"/>
-      <c r="F211" s="3"/>
+      <c r="F211" s="5"/>
       <c r="G211" s="3"/>
       <c r="H211" s="3"/>
       <c r="I211" s="3"/>
@@ -12051,7 +12130,7 @@
       <c r="C212" s="3"/>
       <c r="D212" s="3"/>
       <c r="E212" s="3"/>
-      <c r="F212" s="3"/>
+      <c r="F212" s="5"/>
       <c r="G212" s="3"/>
       <c r="H212" s="3"/>
       <c r="I212" s="3"/>
@@ -12078,7 +12157,7 @@
       <c r="C213" s="3"/>
       <c r="D213" s="3"/>
       <c r="E213" s="3"/>
-      <c r="F213" s="3"/>
+      <c r="F213" s="5"/>
       <c r="G213" s="3"/>
       <c r="H213" s="3"/>
       <c r="I213" s="3"/>
@@ -12105,7 +12184,7 @@
       <c r="C214" s="3"/>
       <c r="D214" s="3"/>
       <c r="E214" s="3"/>
-      <c r="F214" s="3"/>
+      <c r="F214" s="5"/>
       <c r="G214" s="3"/>
       <c r="H214" s="3"/>
       <c r="I214" s="3"/>
@@ -12132,7 +12211,7 @@
       <c r="C215" s="3"/>
       <c r="D215" s="3"/>
       <c r="E215" s="3"/>
-      <c r="F215" s="3"/>
+      <c r="F215" s="5"/>
       <c r="G215" s="3"/>
       <c r="H215" s="3"/>
       <c r="I215" s="3"/>
@@ -12159,7 +12238,7 @@
       <c r="C216" s="3"/>
       <c r="D216" s="3"/>
       <c r="E216" s="3"/>
-      <c r="F216" s="3"/>
+      <c r="F216" s="5"/>
       <c r="G216" s="3"/>
       <c r="H216" s="3"/>
       <c r="I216" s="3"/>
@@ -12186,7 +12265,7 @@
       <c r="C217" s="3"/>
       <c r="D217" s="3"/>
       <c r="E217" s="3"/>
-      <c r="F217" s="3"/>
+      <c r="F217" s="5"/>
       <c r="G217" s="3"/>
       <c r="H217" s="3"/>
       <c r="I217" s="3"/>
@@ -12213,7 +12292,7 @@
       <c r="C218" s="3"/>
       <c r="D218" s="3"/>
       <c r="E218" s="3"/>
-      <c r="F218" s="3"/>
+      <c r="F218" s="5"/>
       <c r="G218" s="3"/>
       <c r="H218" s="3"/>
       <c r="I218" s="3"/>
@@ -12240,7 +12319,7 @@
       <c r="C219" s="3"/>
       <c r="D219" s="3"/>
       <c r="E219" s="3"/>
-      <c r="F219" s="3"/>
+      <c r="F219" s="5"/>
       <c r="G219" s="3"/>
       <c r="H219" s="3"/>
       <c r="I219" s="3"/>
@@ -12267,7 +12346,7 @@
       <c r="C220" s="3"/>
       <c r="D220" s="3"/>
       <c r="E220" s="3"/>
-      <c r="F220" s="3"/>
+      <c r="F220" s="5"/>
       <c r="G220" s="3"/>
       <c r="H220" s="3"/>
       <c r="I220" s="3"/>
@@ -12294,7 +12373,7 @@
       <c r="C221" s="3"/>
       <c r="D221" s="3"/>
       <c r="E221" s="3"/>
-      <c r="F221" s="3"/>
+      <c r="F221" s="5"/>
       <c r="G221" s="3"/>
       <c r="H221" s="3"/>
       <c r="I221" s="3"/>
@@ -12321,7 +12400,7 @@
       <c r="C222" s="3"/>
       <c r="D222" s="3"/>
       <c r="E222" s="3"/>
-      <c r="F222" s="3"/>
+      <c r="F222" s="5"/>
       <c r="G222" s="3"/>
       <c r="H222" s="3"/>
       <c r="I222" s="3"/>
@@ -12348,7 +12427,7 @@
       <c r="C223" s="3"/>
       <c r="D223" s="3"/>
       <c r="E223" s="3"/>
-      <c r="F223" s="3"/>
+      <c r="F223" s="5"/>
       <c r="G223" s="3"/>
       <c r="H223" s="3"/>
       <c r="I223" s="3"/>
@@ -12375,7 +12454,7 @@
       <c r="C224" s="3"/>
       <c r="D224" s="3"/>
       <c r="E224" s="3"/>
-      <c r="F224" s="3"/>
+      <c r="F224" s="5"/>
       <c r="G224" s="3"/>
       <c r="H224" s="3"/>
       <c r="I224" s="3"/>
@@ -12402,7 +12481,7 @@
       <c r="C225" s="3"/>
       <c r="D225" s="3"/>
       <c r="E225" s="3"/>
-      <c r="F225" s="3"/>
+      <c r="F225" s="5"/>
       <c r="G225" s="3"/>
       <c r="H225" s="3"/>
       <c r="I225" s="3"/>
@@ -12429,7 +12508,7 @@
       <c r="C226" s="3"/>
       <c r="D226" s="3"/>
       <c r="E226" s="3"/>
-      <c r="F226" s="3"/>
+      <c r="F226" s="5"/>
       <c r="G226" s="3"/>
       <c r="H226" s="3"/>
       <c r="I226" s="3"/>
@@ -12456,7 +12535,7 @@
       <c r="C227" s="3"/>
       <c r="D227" s="3"/>
       <c r="E227" s="3"/>
-      <c r="F227" s="3"/>
+      <c r="F227" s="5"/>
       <c r="G227" s="3"/>
       <c r="H227" s="3"/>
       <c r="I227" s="3"/>
@@ -12483,7 +12562,7 @@
       <c r="C228" s="3"/>
       <c r="D228" s="3"/>
       <c r="E228" s="3"/>
-      <c r="F228" s="3"/>
+      <c r="F228" s="5"/>
       <c r="G228" s="3"/>
       <c r="H228" s="3"/>
       <c r="I228" s="3"/>
@@ -12510,7 +12589,7 @@
       <c r="C229" s="3"/>
       <c r="D229" s="3"/>
       <c r="E229" s="3"/>
-      <c r="F229" s="3"/>
+      <c r="F229" s="5"/>
       <c r="G229" s="3"/>
       <c r="H229" s="3"/>
       <c r="I229" s="3"/>
@@ -12537,7 +12616,7 @@
       <c r="C230" s="3"/>
       <c r="D230" s="3"/>
       <c r="E230" s="3"/>
-      <c r="F230" s="3"/>
+      <c r="F230" s="5"/>
       <c r="G230" s="3"/>
       <c r="H230" s="3"/>
       <c r="I230" s="3"/>
@@ -12564,7 +12643,7 @@
       <c r="C231" s="3"/>
       <c r="D231" s="3"/>
       <c r="E231" s="3"/>
-      <c r="F231" s="3"/>
+      <c r="F231" s="5"/>
       <c r="G231" s="3"/>
       <c r="H231" s="3"/>
       <c r="I231" s="3"/>
@@ -12591,7 +12670,7 @@
       <c r="C232" s="3"/>
       <c r="D232" s="3"/>
       <c r="E232" s="3"/>
-      <c r="F232" s="3"/>
+      <c r="F232" s="5"/>
       <c r="G232" s="3"/>
       <c r="H232" s="3"/>
       <c r="I232" s="3"/>
@@ -12618,7 +12697,7 @@
       <c r="C233" s="3"/>
       <c r="D233" s="3"/>
       <c r="E233" s="3"/>
-      <c r="F233" s="3"/>
+      <c r="F233" s="5"/>
       <c r="G233" s="3"/>
       <c r="H233" s="3"/>
       <c r="I233" s="3"/>
@@ -12645,7 +12724,7 @@
       <c r="C234" s="3"/>
       <c r="D234" s="3"/>
       <c r="E234" s="3"/>
-      <c r="F234" s="3"/>
+      <c r="F234" s="5"/>
       <c r="G234" s="3"/>
       <c r="H234" s="3"/>
       <c r="I234" s="3"/>
@@ -12672,7 +12751,7 @@
       <c r="C235" s="3"/>
       <c r="D235" s="3"/>
       <c r="E235" s="3"/>
-      <c r="F235" s="3"/>
+      <c r="F235" s="5"/>
       <c r="G235" s="3"/>
       <c r="H235" s="3"/>
       <c r="I235" s="3"/>
@@ -12699,7 +12778,7 @@
       <c r="C236" s="3"/>
       <c r="D236" s="3"/>
       <c r="E236" s="3"/>
-      <c r="F236" s="3"/>
+      <c r="F236" s="5"/>
       <c r="G236" s="3"/>
       <c r="H236" s="3"/>
       <c r="I236" s="3"/>
@@ -12726,7 +12805,7 @@
       <c r="C237" s="3"/>
       <c r="D237" s="3"/>
       <c r="E237" s="3"/>
-      <c r="F237" s="3"/>
+      <c r="F237" s="5"/>
       <c r="G237" s="3"/>
       <c r="H237" s="3"/>
       <c r="I237" s="3"/>
@@ -12753,7 +12832,7 @@
       <c r="C238" s="3"/>
       <c r="D238" s="3"/>
       <c r="E238" s="3"/>
-      <c r="F238" s="3"/>
+      <c r="F238" s="5"/>
       <c r="G238" s="3"/>
       <c r="H238" s="3"/>
       <c r="I238" s="3"/>
@@ -12780,7 +12859,7 @@
       <c r="C239" s="3"/>
       <c r="D239" s="3"/>
       <c r="E239" s="3"/>
-      <c r="F239" s="3"/>
+      <c r="F239" s="5"/>
       <c r="G239" s="3"/>
       <c r="H239" s="3"/>
       <c r="I239" s="3"/>
@@ -12807,7 +12886,7 @@
       <c r="C240" s="3"/>
       <c r="D240" s="3"/>
       <c r="E240" s="3"/>
-      <c r="F240" s="3"/>
+      <c r="F240" s="5"/>
       <c r="G240" s="3"/>
       <c r="H240" s="3"/>
       <c r="I240" s="3"/>
@@ -12834,7 +12913,7 @@
       <c r="C241" s="3"/>
       <c r="D241" s="3"/>
       <c r="E241" s="3"/>
-      <c r="F241" s="3"/>
+      <c r="F241" s="5"/>
       <c r="G241" s="3"/>
       <c r="H241" s="3"/>
       <c r="I241" s="3"/>
@@ -12861,7 +12940,7 @@
       <c r="C242" s="3"/>
       <c r="D242" s="3"/>
       <c r="E242" s="3"/>
-      <c r="F242" s="3"/>
+      <c r="F242" s="5"/>
       <c r="G242" s="3"/>
       <c r="H242" s="3"/>
       <c r="I242" s="3"/>
@@ -12888,7 +12967,7 @@
       <c r="C243" s="3"/>
       <c r="D243" s="3"/>
       <c r="E243" s="3"/>
-      <c r="F243" s="3"/>
+      <c r="F243" s="5"/>
       <c r="G243" s="3"/>
       <c r="H243" s="3"/>
       <c r="I243" s="3"/>
@@ -12915,7 +12994,7 @@
       <c r="C244" s="3"/>
       <c r="D244" s="3"/>
       <c r="E244" s="3"/>
-      <c r="F244" s="3"/>
+      <c r="F244" s="5"/>
       <c r="G244" s="3"/>
       <c r="H244" s="3"/>
       <c r="I244" s="3"/>
@@ -12942,7 +13021,7 @@
       <c r="C245" s="3"/>
       <c r="D245" s="3"/>
       <c r="E245" s="3"/>
-      <c r="F245" s="3"/>
+      <c r="F245" s="5"/>
       <c r="G245" s="3"/>
       <c r="H245" s="3"/>
       <c r="I245" s="3"/>
@@ -12969,7 +13048,7 @@
       <c r="C246" s="3"/>
       <c r="D246" s="3"/>
       <c r="E246" s="3"/>
-      <c r="F246" s="3"/>
+      <c r="F246" s="5"/>
       <c r="G246" s="3"/>
       <c r="H246" s="3"/>
       <c r="I246" s="3"/>
@@ -12996,7 +13075,7 @@
       <c r="C247" s="3"/>
       <c r="D247" s="3"/>
       <c r="E247" s="3"/>
-      <c r="F247" s="3"/>
+      <c r="F247" s="5"/>
       <c r="G247" s="3"/>
       <c r="H247" s="3"/>
       <c r="I247" s="3"/>
@@ -13023,7 +13102,7 @@
       <c r="C248" s="3"/>
       <c r="D248" s="3"/>
       <c r="E248" s="3"/>
-      <c r="F248" s="3"/>
+      <c r="F248" s="5"/>
       <c r="G248" s="3"/>
       <c r="H248" s="3"/>
       <c r="I248" s="3"/>
@@ -13050,7 +13129,7 @@
       <c r="C249" s="3"/>
       <c r="D249" s="3"/>
       <c r="E249" s="3"/>
-      <c r="F249" s="3"/>
+      <c r="F249" s="5"/>
       <c r="G249" s="3"/>
       <c r="H249" s="3"/>
       <c r="I249" s="3"/>
@@ -13077,7 +13156,7 @@
       <c r="C250" s="3"/>
       <c r="D250" s="3"/>
       <c r="E250" s="3"/>
-      <c r="F250" s="3"/>
+      <c r="F250" s="5"/>
       <c r="G250" s="3"/>
       <c r="H250" s="3"/>
       <c r="I250" s="3"/>
@@ -13104,7 +13183,7 @@
       <c r="C251" s="3"/>
       <c r="D251" s="3"/>
       <c r="E251" s="3"/>
-      <c r="F251" s="3"/>
+      <c r="F251" s="5"/>
       <c r="G251" s="3"/>
       <c r="H251" s="3"/>
       <c r="I251" s="3"/>
@@ -13131,7 +13210,7 @@
       <c r="C252" s="3"/>
       <c r="D252" s="3"/>
       <c r="E252" s="3"/>
-      <c r="F252" s="3"/>
+      <c r="F252" s="5"/>
       <c r="G252" s="3"/>
       <c r="H252" s="3"/>
       <c r="I252" s="3"/>
@@ -13158,7 +13237,7 @@
       <c r="C253" s="3"/>
       <c r="D253" s="3"/>
       <c r="E253" s="3"/>
-      <c r="F253" s="3"/>
+      <c r="F253" s="5"/>
       <c r="G253" s="3"/>
       <c r="H253" s="3"/>
       <c r="I253" s="3"/>
@@ -13185,7 +13264,7 @@
       <c r="C254" s="3"/>
       <c r="D254" s="3"/>
       <c r="E254" s="3"/>
-      <c r="F254" s="3"/>
+      <c r="F254" s="5"/>
       <c r="G254" s="3"/>
       <c r="H254" s="3"/>
       <c r="I254" s="3"/>
@@ -13212,7 +13291,7 @@
       <c r="C255" s="3"/>
       <c r="D255" s="3"/>
       <c r="E255" s="3"/>
-      <c r="F255" s="3"/>
+      <c r="F255" s="5"/>
       <c r="G255" s="3"/>
       <c r="H255" s="3"/>
       <c r="I255" s="3"/>
@@ -13239,7 +13318,7 @@
       <c r="C256" s="3"/>
       <c r="D256" s="3"/>
       <c r="E256" s="3"/>
-      <c r="F256" s="3"/>
+      <c r="F256" s="5"/>
       <c r="G256" s="3"/>
       <c r="H256" s="3"/>
       <c r="I256" s="3"/>
@@ -13266,7 +13345,7 @@
       <c r="C257" s="3"/>
       <c r="D257" s="3"/>
       <c r="E257" s="3"/>
-      <c r="F257" s="3"/>
+      <c r="F257" s="5"/>
       <c r="G257" s="3"/>
       <c r="H257" s="3"/>
       <c r="I257" s="3"/>
@@ -13293,7 +13372,7 @@
       <c r="C258" s="3"/>
       <c r="D258" s="3"/>
       <c r="E258" s="3"/>
-      <c r="F258" s="3"/>
+      <c r="F258" s="5"/>
       <c r="G258" s="3"/>
       <c r="H258" s="3"/>
       <c r="I258" s="3"/>
@@ -13320,7 +13399,7 @@
       <c r="C259" s="3"/>
       <c r="D259" s="3"/>
       <c r="E259" s="3"/>
-      <c r="F259" s="3"/>
+      <c r="F259" s="5"/>
       <c r="G259" s="3"/>
       <c r="H259" s="3"/>
       <c r="I259" s="3"/>
@@ -13347,7 +13426,7 @@
       <c r="C260" s="3"/>
       <c r="D260" s="3"/>
       <c r="E260" s="3"/>
-      <c r="F260" s="3"/>
+      <c r="F260" s="5"/>
       <c r="G260" s="3"/>
       <c r="H260" s="3"/>
       <c r="I260" s="3"/>
@@ -13374,7 +13453,7 @@
       <c r="C261" s="3"/>
       <c r="D261" s="3"/>
       <c r="E261" s="3"/>
-      <c r="F261" s="3"/>
+      <c r="F261" s="5"/>
       <c r="G261" s="3"/>
       <c r="H261" s="3"/>
       <c r="I261" s="3"/>
@@ -13401,7 +13480,7 @@
       <c r="C262" s="3"/>
       <c r="D262" s="3"/>
       <c r="E262" s="3"/>
-      <c r="F262" s="3"/>
+      <c r="F262" s="5"/>
       <c r="G262" s="3"/>
       <c r="H262" s="3"/>
       <c r="I262" s="3"/>
@@ -13428,7 +13507,7 @@
       <c r="C263" s="3"/>
       <c r="D263" s="3"/>
       <c r="E263" s="3"/>
-      <c r="F263" s="3"/>
+      <c r="F263" s="5"/>
       <c r="G263" s="3"/>
       <c r="H263" s="3"/>
       <c r="I263" s="3"/>
@@ -13455,7 +13534,7 @@
       <c r="C264" s="3"/>
       <c r="D264" s="3"/>
       <c r="E264" s="3"/>
-      <c r="F264" s="3"/>
+      <c r="F264" s="5"/>
       <c r="G264" s="3"/>
       <c r="H264" s="3"/>
       <c r="I264" s="3"/>
@@ -13482,7 +13561,7 @@
       <c r="C265" s="3"/>
       <c r="D265" s="3"/>
       <c r="E265" s="3"/>
-      <c r="F265" s="3"/>
+      <c r="F265" s="5"/>
       <c r="G265" s="3"/>
       <c r="H265" s="3"/>
       <c r="I265" s="3"/>
@@ -13509,7 +13588,7 @@
       <c r="C266" s="3"/>
       <c r="D266" s="3"/>
       <c r="E266" s="3"/>
-      <c r="F266" s="3"/>
+      <c r="F266" s="5"/>
       <c r="G266" s="3"/>
       <c r="H266" s="3"/>
       <c r="I266" s="3"/>
@@ -13536,7 +13615,7 @@
       <c r="C267" s="3"/>
       <c r="D267" s="3"/>
       <c r="E267" s="3"/>
-      <c r="F267" s="3"/>
+      <c r="F267" s="5"/>
       <c r="G267" s="3"/>
       <c r="H267" s="3"/>
       <c r="I267" s="3"/>
@@ -13563,7 +13642,7 @@
       <c r="C268" s="3"/>
       <c r="D268" s="3"/>
       <c r="E268" s="3"/>
-      <c r="F268" s="3"/>
+      <c r="F268" s="5"/>
       <c r="G268" s="3"/>
       <c r="H268" s="3"/>
       <c r="I268" s="3"/>
@@ -13590,7 +13669,7 @@
       <c r="C269" s="3"/>
       <c r="D269" s="3"/>
       <c r="E269" s="3"/>
-      <c r="F269" s="3"/>
+      <c r="F269" s="5"/>
       <c r="G269" s="3"/>
       <c r="H269" s="3"/>
       <c r="I269" s="3"/>
@@ -13617,7 +13696,7 @@
       <c r="C270" s="3"/>
       <c r="D270" s="3"/>
       <c r="E270" s="3"/>
-      <c r="F270" s="3"/>
+      <c r="F270" s="5"/>
       <c r="G270" s="3"/>
       <c r="H270" s="3"/>
       <c r="I270" s="3"/>
@@ -13644,7 +13723,7 @@
       <c r="C271" s="3"/>
       <c r="D271" s="3"/>
       <c r="E271" s="3"/>
-      <c r="F271" s="3"/>
+      <c r="F271" s="5"/>
       <c r="G271" s="3"/>
       <c r="H271" s="3"/>
       <c r="I271" s="3"/>
@@ -13671,7 +13750,7 @@
       <c r="C272" s="3"/>
       <c r="D272" s="3"/>
       <c r="E272" s="3"/>
-      <c r="F272" s="3"/>
+      <c r="F272" s="5"/>
       <c r="G272" s="3"/>
       <c r="H272" s="3"/>
       <c r="I272" s="3"/>
@@ -13698,7 +13777,7 @@
       <c r="C273" s="3"/>
       <c r="D273" s="3"/>
       <c r="E273" s="3"/>
-      <c r="F273" s="3"/>
+      <c r="F273" s="5"/>
       <c r="G273" s="3"/>
       <c r="H273" s="3"/>
       <c r="I273" s="3"/>
@@ -13725,7 +13804,7 @@
       <c r="C274" s="3"/>
       <c r="D274" s="3"/>
       <c r="E274" s="3"/>
-      <c r="F274" s="3"/>
+      <c r="F274" s="5"/>
       <c r="G274" s="3"/>
       <c r="H274" s="3"/>
       <c r="I274" s="3"/>
@@ -13752,7 +13831,7 @@
       <c r="C275" s="3"/>
       <c r="D275" s="3"/>
       <c r="E275" s="3"/>
-      <c r="F275" s="3"/>
+      <c r="F275" s="5"/>
       <c r="G275" s="3"/>
       <c r="H275" s="3"/>
       <c r="I275" s="3"/>
@@ -13779,7 +13858,7 @@
       <c r="C276" s="3"/>
       <c r="D276" s="3"/>
       <c r="E276" s="3"/>
-      <c r="F276" s="3"/>
+      <c r="F276" s="5"/>
       <c r="G276" s="3"/>
       <c r="H276" s="3"/>
       <c r="I276" s="3"/>
@@ -13806,7 +13885,7 @@
       <c r="C277" s="3"/>
       <c r="D277" s="3"/>
       <c r="E277" s="3"/>
-      <c r="F277" s="3"/>
+      <c r="F277" s="5"/>
       <c r="G277" s="3"/>
       <c r="H277" s="3"/>
       <c r="I277" s="3"/>
@@ -13833,7 +13912,7 @@
       <c r="C278" s="3"/>
       <c r="D278" s="3"/>
       <c r="E278" s="3"/>
-      <c r="F278" s="3"/>
+      <c r="F278" s="5"/>
       <c r="G278" s="3"/>
       <c r="H278" s="3"/>
       <c r="I278" s="3"/>
@@ -13860,7 +13939,7 @@
       <c r="C279" s="3"/>
       <c r="D279" s="3"/>
       <c r="E279" s="3"/>
-      <c r="F279" s="3"/>
+      <c r="F279" s="5"/>
       <c r="G279" s="3"/>
       <c r="H279" s="3"/>
       <c r="I279" s="3"/>
@@ -13887,7 +13966,7 @@
       <c r="C280" s="3"/>
       <c r="D280" s="3"/>
       <c r="E280" s="3"/>
-      <c r="F280" s="3"/>
+      <c r="F280" s="5"/>
       <c r="G280" s="3"/>
       <c r="H280" s="3"/>
       <c r="I280" s="3"/>
@@ -13914,7 +13993,7 @@
       <c r="C281" s="3"/>
       <c r="D281" s="3"/>
       <c r="E281" s="3"/>
-      <c r="F281" s="3"/>
+      <c r="F281" s="5"/>
       <c r="G281" s="3"/>
       <c r="H281" s="3"/>
       <c r="I281" s="3"/>
@@ -13941,7 +14020,7 @@
       <c r="C282" s="3"/>
       <c r="D282" s="3"/>
       <c r="E282" s="3"/>
-      <c r="F282" s="3"/>
+      <c r="F282" s="5"/>
       <c r="G282" s="3"/>
       <c r="H282" s="3"/>
       <c r="I282" s="3"/>
@@ -13968,7 +14047,7 @@
       <c r="C283" s="3"/>
       <c r="D283" s="3"/>
       <c r="E283" s="3"/>
-      <c r="F283" s="3"/>
+      <c r="F283" s="5"/>
       <c r="G283" s="3"/>
       <c r="H283" s="3"/>
       <c r="I283" s="3"/>
@@ -13995,7 +14074,7 @@
       <c r="C284" s="3"/>
       <c r="D284" s="3"/>
       <c r="E284" s="3"/>
-      <c r="F284" s="3"/>
+      <c r="F284" s="5"/>
       <c r="G284" s="3"/>
       <c r="H284" s="3"/>
       <c r="I284" s="3"/>
@@ -14022,7 +14101,7 @@
       <c r="C285" s="3"/>
       <c r="D285" s="3"/>
       <c r="E285" s="3"/>
-      <c r="F285" s="3"/>
+      <c r="F285" s="5"/>
       <c r="G285" s="3"/>
       <c r="H285" s="3"/>
       <c r="I285" s="3"/>
@@ -14049,7 +14128,7 @@
       <c r="C286" s="3"/>
       <c r="D286" s="3"/>
       <c r="E286" s="3"/>
-      <c r="F286" s="3"/>
+      <c r="F286" s="5"/>
       <c r="G286" s="3"/>
       <c r="H286" s="3"/>
       <c r="I286" s="3"/>
@@ -14076,7 +14155,7 @@
       <c r="C287" s="3"/>
       <c r="D287" s="3"/>
       <c r="E287" s="3"/>
-      <c r="F287" s="3"/>
+      <c r="F287" s="5"/>
       <c r="G287" s="3"/>
       <c r="H287" s="3"/>
       <c r="I287" s="3"/>
@@ -14103,7 +14182,7 @@
       <c r="C288" s="3"/>
       <c r="D288" s="3"/>
       <c r="E288" s="3"/>
-      <c r="F288" s="3"/>
+      <c r="F288" s="5"/>
       <c r="G288" s="3"/>
       <c r="H288" s="3"/>
       <c r="I288" s="3"/>
@@ -14130,7 +14209,7 @@
       <c r="C289" s="3"/>
       <c r="D289" s="3"/>
       <c r="E289" s="3"/>
-      <c r="F289" s="3"/>
+      <c r="F289" s="5"/>
       <c r="G289" s="3"/>
       <c r="H289" s="3"/>
       <c r="I289" s="3"/>
@@ -14157,7 +14236,7 @@
       <c r="C290" s="3"/>
       <c r="D290" s="3"/>
       <c r="E290" s="3"/>
-      <c r="F290" s="3"/>
+      <c r="F290" s="5"/>
       <c r="G290" s="3"/>
       <c r="H290" s="3"/>
       <c r="I290" s="3"/>
@@ -14184,7 +14263,7 @@
       <c r="C291" s="3"/>
       <c r="D291" s="3"/>
       <c r="E291" s="3"/>
-      <c r="F291" s="3"/>
+      <c r="F291" s="5"/>
       <c r="G291" s="3"/>
       <c r="H291" s="3"/>
       <c r="I291" s="3"/>
@@ -14211,7 +14290,7 @@
       <c r="C292" s="3"/>
       <c r="D292" s="3"/>
       <c r="E292" s="3"/>
-      <c r="F292" s="3"/>
+      <c r="F292" s="5"/>
       <c r="G292" s="3"/>
       <c r="H292" s="3"/>
       <c r="I292" s="3"/>
@@ -14238,7 +14317,7 @@
       <c r="C293" s="3"/>
       <c r="D293" s="3"/>
       <c r="E293" s="3"/>
-      <c r="F293" s="3"/>
+      <c r="F293" s="5"/>
       <c r="G293" s="3"/>
       <c r="H293" s="3"/>
       <c r="I293" s="3"/>
@@ -14265,7 +14344,7 @@
       <c r="C294" s="3"/>
       <c r="D294" s="3"/>
       <c r="E294" s="3"/>
-      <c r="F294" s="3"/>
+      <c r="F294" s="5"/>
       <c r="G294" s="3"/>
       <c r="H294" s="3"/>
       <c r="I294" s="3"/>
@@ -14292,7 +14371,7 @@
       <c r="C295" s="3"/>
       <c r="D295" s="3"/>
       <c r="E295" s="3"/>
-      <c r="F295" s="3"/>
+      <c r="F295" s="5"/>
       <c r="G295" s="3"/>
       <c r="H295" s="3"/>
       <c r="I295" s="3"/>
@@ -14319,7 +14398,7 @@
       <c r="C296" s="3"/>
       <c r="D296" s="3"/>
       <c r="E296" s="3"/>
-      <c r="F296" s="3"/>
+      <c r="F296" s="5"/>
       <c r="G296" s="3"/>
       <c r="H296" s="3"/>
       <c r="I296" s="3"/>
@@ -14346,7 +14425,7 @@
       <c r="C297" s="3"/>
       <c r="D297" s="3"/>
       <c r="E297" s="3"/>
-      <c r="F297" s="3"/>
+      <c r="F297" s="5"/>
       <c r="G297" s="3"/>
       <c r="H297" s="3"/>
       <c r="I297" s="3"/>
@@ -14373,7 +14452,7 @@
       <c r="C298" s="3"/>
       <c r="D298" s="3"/>
       <c r="E298" s="3"/>
-      <c r="F298" s="3"/>
+      <c r="F298" s="5"/>
       <c r="G298" s="3"/>
       <c r="H298" s="3"/>
       <c r="I298" s="3"/>
@@ -14400,7 +14479,7 @@
       <c r="C299" s="3"/>
       <c r="D299" s="3"/>
       <c r="E299" s="3"/>
-      <c r="F299" s="3"/>
+      <c r="F299" s="5"/>
       <c r="G299" s="3"/>
       <c r="H299" s="3"/>
       <c r="I299" s="3"/>
@@ -14427,7 +14506,7 @@
       <c r="C300" s="3"/>
       <c r="D300" s="3"/>
       <c r="E300" s="3"/>
-      <c r="F300" s="3"/>
+      <c r="F300" s="5"/>
       <c r="G300" s="3"/>
       <c r="H300" s="3"/>
       <c r="I300" s="3"/>
@@ -22542,19 +22621,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F500">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>F2="REUSE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>F2="REFACTOR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>F2="REPLACE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="4" priority="4">
       <formula>F2="REMOVE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="3" priority="5">
       <formula>F2="INVESTIGATE"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Record CMake change commit in traceability register
</commit_message>
<xml_diff>
--- a/planning/traceability/MOHID-NG_Traceability_Register.xlsx
+++ b/planning/traceability/MOHID-NG_Traceability_Register.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04-Test\home\jflavio\Programas\MohidNG\planning\traceability\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6410E2F-2F10-47BD-AF1A-9C89167E39EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9487F70E-72D3-4E9A-A5F6-5CDE4BAC0EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="593">
   <si>
     <t>MOHID-NG Traceability and Change-Management Register</t>
   </si>
@@ -1820,6 +1820,9 @@
   </si>
   <si>
     <t>Alteração restrita ao sistema de build, realizada com assistência do Codex a pedido do mantenedor. Não modifica modelos científicos, métodos numéricos ou comportamento funcional. Eventuais ganhos de desempenho dependem das configurações de compilação e ainda não foram verificados por benchmark.</t>
+  </si>
+  <si>
+    <t>30c26c2876d91ac1b1440d0c32953fc9c8dcd5c8</t>
   </si>
 </sst>
 </file>
@@ -1967,6 +1970,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1985,23 +1991,11 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="49">
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2151,6 +2145,15 @@
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2422,27 +2425,27 @@
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Data" dataDxfId="45"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Título" dataDxfId="44"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Categoria" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Status" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Prioridade" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Responsável" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Fonte/Justificativa" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="REQ_IDs" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ADR_IDs" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Arquivos/paths" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Resumo da alteração" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Razão" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Testes/Gates" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="EVID_IDs" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Branch" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Commit" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="PR" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Release" dataDxfId="31"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Impacto científico" dataDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Impacto numérico" dataDxfId="29"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Impacto API/ABI" dataDxfId="28"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0100-000017000000}" name="Documentação atualizada" dataDxfId="27"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0100-000018000000}" name="Compatibilidade/risco" dataDxfId="26"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0100-000019000000}" name="Observações" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Status" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Prioridade" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Responsável" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Fonte/Justificativa" dataDxfId="39"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="REQ_IDs" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ADR_IDs" dataDxfId="37"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Arquivos/paths" dataDxfId="36"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Resumo da alteração" dataDxfId="35"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Razão" dataDxfId="34"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Testes/Gates" dataDxfId="33"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="EVID_IDs" dataDxfId="32"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Branch" dataDxfId="31"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Commit" dataDxfId="30"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="PR" dataDxfId="29"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Release" dataDxfId="28"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Impacto científico" dataDxfId="27"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Impacto numérico" dataDxfId="26"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Impacto API/ABI" dataDxfId="25"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0100-000017000000}" name="Documentação atualizada" dataDxfId="24"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0100-000018000000}" name="Compatibilidade/risco" dataDxfId="23"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0100-000019000000}" name="Observações" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2473,17 +2476,17 @@
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="RequirementsTable" displayName="RequirementsTable" ref="A1:L60" totalsRowShown="0">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="REQ_ID" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Tipo" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Título" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="REQ_ID" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Tipo" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Título" dataDxfId="19"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Texto normativo"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Estado v0.14" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Fonte" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="ADR_IDs" dataDxfId="19"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="CHG_IDs" dataDxfId="18"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="TEST/Gate_IDs" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="EVID_IDs" dataDxfId="16"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Status implementação" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Estado v0.14" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Fonte" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="ADR_IDs" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="CHG_IDs" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="TEST/Gate_IDs" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="EVID_IDs" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Status implementação" dataDxfId="12"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="Observações"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2495,15 +2498,15 @@
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Record_ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Tipo"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Decisão/Título" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Status" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Fonte" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Decisão/Título" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Status" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Fonte" dataDxfId="9"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="REQ_IDs"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="ADR_file"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Supersedes"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Racional/Evidência"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" name="Responsável"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Data decisão" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Data decisão" dataDxfId="8"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" name="Observações"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2774,16 +2777,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2"/>
@@ -2932,16 +2935,16 @@
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="15">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="5" t="s">
@@ -3094,38 +3097,38 @@
       <c r="H24" s="2"/>
     </row>
     <row r="25" spans="1:8" ht="15">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="23" t="s">
+      <c r="A26" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
-      <c r="H26" s="23"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="2"/>
@@ -3138,58 +3141,58 @@
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:8" ht="15">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="22"/>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
-      <c r="H30" s="20"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="20"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20"/>
+      <c r="A31" s="21"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="20"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20"/>
+      <c r="A32" s="21"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="20"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
+      <c r="A33" s="21"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -5250,38 +5253,38 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="21" t="s">
         <v>566</v>
       </c>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="20"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="20"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5303,16 +5306,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="3" spans="1:8" ht="15">
       <c r="A3" s="1" t="s">
@@ -5418,68 +5421,68 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="15">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="21"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="20"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="20"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="21"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6245,13 +6248,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D100">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>D2="Concluído"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>D2="Em andamento"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="3">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>D2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6276,7 +6279,7 @@
     <col min="3" max="3" width="34" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="10" style="26" customWidth="1"/>
+    <col min="6" max="6" width="10" style="20" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="32" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
@@ -6287,7 +6290,7 @@
     <col min="14" max="14" width="30" customWidth="1"/>
     <col min="15" max="15" width="27.875" customWidth="1"/>
     <col min="16" max="16" width="24" customWidth="1"/>
-    <col min="17" max="17" width="40" customWidth="1"/>
+    <col min="17" max="17" width="42.875" customWidth="1"/>
     <col min="18" max="18" width="16" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
     <col min="20" max="22" width="16" customWidth="1"/>
@@ -6486,7 +6489,9 @@
       <c r="P3" s="8" t="s">
         <v>588</v>
       </c>
-      <c r="Q3" s="8"/>
+      <c r="Q3" s="8" t="s">
+        <v>592</v>
+      </c>
       <c r="R3" s="13"/>
       <c r="S3" s="8"/>
       <c r="T3" s="8" t="s">
@@ -22621,19 +22626,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F500">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>F2="REUSE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>F2="REFACTOR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>F2="REPLACE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>F2="REMOVE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>F2="INVESTIGATE"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>